<commit_message>
#18 Client and eSpark BOM updated acc to Design
</commit_message>
<xml_diff>
--- a/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
+++ b/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="232">
   <si>
     <t>Component list</t>
   </si>
@@ -252,9 +252,6 @@
     <t>PCI Express Mini Card (Mini PCIe)</t>
   </si>
   <si>
-    <t>CONN MOD JACK 8P8C R/A SHIELDED</t>
-  </si>
-  <si>
     <t>33uH 2.3A ±20% SMD,6.6x7.3mm Inductors</t>
   </si>
   <si>
@@ -318,9 +315,6 @@
     <t>RES SMD 12.4K OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>IC POE CNTRL 1 CHANNEL 8TSSOP</t>
-  </si>
-  <si>
     <t>Step-down type SOIC-8-EP DC-DC Converters ROHS</t>
   </si>
   <si>
@@ -363,9 +357,6 @@
     <t>Mini PCIE Pad</t>
   </si>
   <si>
-    <t>RJE73-188-00441</t>
-  </si>
-  <si>
     <t>SOT-723</t>
   </si>
   <si>
@@ -384,9 +375,6 @@
     <t>Res-0603</t>
   </si>
   <si>
-    <t>8-TSSOP</t>
-  </si>
-  <si>
     <t>8-SOIC-EP</t>
   </si>
   <si>
@@ -504,9 +492,6 @@
     <t>RC0603FR-0712K4L</t>
   </si>
   <si>
-    <t>TPS2375PW-1</t>
-  </si>
-  <si>
     <t>TX4138</t>
   </si>
   <si>
@@ -549,9 +534,6 @@
     <t>Taiyo Yuden</t>
   </si>
   <si>
-    <t>Amphenol Commercial</t>
-  </si>
-  <si>
     <t>KOHERelec</t>
   </si>
   <si>
@@ -712,6 +694,27 @@
   </si>
   <si>
     <t>Custom Supplier</t>
+  </si>
+  <si>
+    <t>CONN JACK 1PORT 100 BASE-T PCB</t>
+  </si>
+  <si>
+    <t>ARJM11D7-114-AB-EW2</t>
+  </si>
+  <si>
+    <t>Abracon</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>IC POE CNTRL 1 CHANNEL 8SOIC</t>
+  </si>
+  <si>
+    <t>SOIC-8</t>
+  </si>
+  <si>
+    <t>TPS2375DR</t>
   </si>
 </sst>
 </file>
@@ -1259,6 +1262,48 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1267,48 +1312,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1680,13 +1683,13 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="54"/>
-      <c r="O1" s="54"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
     </row>
     <row r="2" spans="1:15" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1697,7 +1700,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="50" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1718,7 +1721,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="51" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1728,7 +1731,7 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
-      <c r="O3" s="55"/>
+      <c r="O3" s="69"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1739,7 +1742,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="52" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1749,7 +1752,7 @@
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
-      <c r="O4" s="56"/>
+      <c r="O4" s="70"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1770,7 +1773,7 @@
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
-      <c r="O5" s="56"/>
+      <c r="O5" s="70"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1787,7 +1790,7 @@
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
-      <c r="O6" s="56"/>
+      <c r="O6" s="70"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1804,7 +1807,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
-      <c r="O7" s="56"/>
+      <c r="O7" s="70"/>
     </row>
     <row r="8" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1821,7 +1824,7 @@
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
-      <c r="O8" s="56"/>
+      <c r="O8" s="70"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1838,43 +1841,43 @@
         <v>61</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="K9" s="29" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="L9" s="29" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="M9" s="29" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="N9" s="29" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="O9" s="29" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="57">
+      <c r="B10" s="54">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="36" t="s">
@@ -1884,16 +1887,16 @@
         <v>62</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="J10" s="36">
         <v>10</v>
@@ -1902,13 +1905,13 @@
         <f>J10*5</f>
         <v>50</v>
       </c>
-      <c r="L10" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M10" s="64">
+      <c r="L10" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M10" s="61">
         <v>1.26E-2</v>
       </c>
-      <c r="N10" s="64">
+      <c r="N10" s="61">
         <f>M10*K10</f>
         <v>0.63</v>
       </c>
@@ -1916,11 +1919,11 @@
     </row>
     <row r="11" spans="1:15" ht="36" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="59">
+      <c r="B11" s="56">
         <f t="shared" ref="B11:B51" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="60" t="s">
+      <c r="C11" s="57" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="38" t="s">
@@ -1930,16 +1933,16 @@
         <v>63</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="J11" s="38">
         <v>1</v>
@@ -1948,24 +1951,24 @@
         <f t="shared" ref="K11" si="1">J11*5</f>
         <v>5</v>
       </c>
-      <c r="L11" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M11" s="65" t="s">
-        <v>218</v>
-      </c>
-      <c r="N11" s="65" t="s">
-        <v>218</v>
+      <c r="L11" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M11" s="62" t="s">
+        <v>212</v>
+      </c>
+      <c r="N11" s="62" t="s">
+        <v>212</v>
       </c>
       <c r="O11" s="38"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="57">
+      <c r="B12" s="54">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="60" t="s">
+      <c r="C12" s="57" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="36" t="s">
@@ -1975,16 +1978,16 @@
         <v>64</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="G12" s="69" t="s">
-        <v>128</v>
+        <v>105</v>
+      </c>
+      <c r="G12" s="66" t="s">
+        <v>124</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="J12" s="36">
         <v>3</v>
@@ -1993,13 +1996,13 @@
         <f>J12*5</f>
         <v>15</v>
       </c>
-      <c r="L12" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M12" s="64">
+      <c r="L12" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M12" s="61">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N12" s="64">
+      <c r="N12" s="61">
         <f>M12*K12</f>
         <v>1.0649999999999999</v>
       </c>
@@ -2007,11 +2010,11 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="59">
+      <c r="B13" s="56">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="60" t="s">
+      <c r="C13" s="57" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="38" t="s">
@@ -2021,16 +2024,16 @@
         <v>65</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="G13" s="70" t="s">
-        <v>129</v>
+        <v>106</v>
+      </c>
+      <c r="G13" s="67" t="s">
+        <v>125</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="J13" s="38">
         <v>1</v>
@@ -2039,13 +2042,13 @@
         <f t="shared" ref="K13" si="2">J13*5</f>
         <v>5</v>
       </c>
-      <c r="L13" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M13" s="65">
+      <c r="L13" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M13" s="62">
         <v>2.33</v>
       </c>
-      <c r="N13" s="65">
+      <c r="N13" s="62">
         <f t="shared" ref="N13" si="3">M13*K13</f>
         <v>11.65</v>
       </c>
@@ -2053,11 +2056,11 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="57">
+      <c r="B14" s="54">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="58" t="s">
+      <c r="C14" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="36" t="s">
@@ -2067,16 +2070,16 @@
         <v>66</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>105</v>
-      </c>
-      <c r="G14" s="69" t="s">
-        <v>130</v>
+        <v>103</v>
+      </c>
+      <c r="G14" s="66" t="s">
+        <v>126</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="J14" s="36">
         <v>1</v>
@@ -2085,13 +2088,13 @@
         <f>J14*5</f>
         <v>5</v>
       </c>
-      <c r="L14" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M14" s="64">
+      <c r="L14" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M14" s="61">
         <v>0.1</v>
       </c>
-      <c r="N14" s="64">
+      <c r="N14" s="61">
         <f>M14*K14</f>
         <v>0.5</v>
       </c>
@@ -2099,11 +2102,11 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="59">
+      <c r="B15" s="56">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="60" t="s">
+      <c r="C15" s="57" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="38" t="s">
@@ -2113,16 +2116,16 @@
         <v>67</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="G15" s="69" t="s">
-        <v>131</v>
+        <v>103</v>
+      </c>
+      <c r="G15" s="66" t="s">
+        <v>127</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="J15" s="38">
         <v>3</v>
@@ -2131,13 +2134,13 @@
         <f t="shared" ref="K15" si="4">J15*5</f>
         <v>15</v>
       </c>
-      <c r="L15" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M15" s="65">
+      <c r="L15" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M15" s="62">
         <v>5.5E-2</v>
       </c>
-      <c r="N15" s="65">
+      <c r="N15" s="62">
         <f t="shared" ref="N15" si="5">M15*K15</f>
         <v>0.82499999999999996</v>
       </c>
@@ -2145,11 +2148,11 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="57">
+      <c r="B16" s="54">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="36" t="s">
@@ -2159,16 +2162,16 @@
         <v>68</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="G16" s="69" t="s">
-        <v>132</v>
+        <v>105</v>
+      </c>
+      <c r="G16" s="66" t="s">
+        <v>128</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="J16" s="36">
         <v>1</v>
@@ -2177,13 +2180,13 @@
         <f>J16*5</f>
         <v>5</v>
       </c>
-      <c r="L16" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M16" s="64">
+      <c r="L16" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M16" s="61">
         <v>0.75</v>
       </c>
-      <c r="N16" s="64">
+      <c r="N16" s="61">
         <f>M16*K16</f>
         <v>3.75</v>
       </c>
@@ -2191,11 +2194,11 @@
     </row>
     <row r="17" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="59">
+      <c r="B17" s="56">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="60" t="s">
+      <c r="C17" s="57" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="38" t="s">
@@ -2205,16 +2208,16 @@
         <v>69</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>107</v>
-      </c>
-      <c r="G17" s="70" t="s">
-        <v>133</v>
+        <v>105</v>
+      </c>
+      <c r="G17" s="67" t="s">
+        <v>129</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="J17" s="38">
         <v>2</v>
@@ -2223,24 +2226,24 @@
         <f t="shared" ref="K17" si="6">J17*5</f>
         <v>10</v>
       </c>
-      <c r="L17" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M17" s="65" t="s">
-        <v>218</v>
-      </c>
-      <c r="N17" s="65" t="s">
-        <v>218</v>
+      <c r="L17" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M17" s="62" t="s">
+        <v>212</v>
+      </c>
+      <c r="N17" s="62" t="s">
+        <v>212</v>
       </c>
       <c r="O17" s="38"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="57">
+      <c r="B18" s="54">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="58" t="s">
+      <c r="C18" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="36" t="s">
@@ -2250,16 +2253,16 @@
         <v>70</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="G18" s="69" t="s">
-        <v>134</v>
+        <v>105</v>
+      </c>
+      <c r="G18" s="66" t="s">
+        <v>130</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="J18" s="36">
         <v>2</v>
@@ -2268,13 +2271,13 @@
         <f>J18*5</f>
         <v>10</v>
       </c>
-      <c r="L18" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M18" s="64">
+      <c r="L18" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M18" s="61">
         <v>9.7000000000000003E-2</v>
       </c>
-      <c r="N18" s="64">
+      <c r="N18" s="61">
         <f>M18*K18</f>
         <v>0.97</v>
       </c>
@@ -2282,11 +2285,11 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="59">
+      <c r="B19" s="56">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="58" t="s">
+      <c r="C19" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="38" t="s">
@@ -2296,16 +2299,16 @@
         <v>71</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>107</v>
-      </c>
-      <c r="G19" s="70" t="s">
-        <v>135</v>
+        <v>105</v>
+      </c>
+      <c r="G19" s="67" t="s">
+        <v>131</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="J19" s="38">
         <v>1</v>
@@ -2314,13 +2317,13 @@
         <f t="shared" ref="K19" si="7">J19*5</f>
         <v>5</v>
       </c>
-      <c r="L19" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M19" s="65">
+      <c r="L19" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M19" s="62">
         <v>0.32</v>
       </c>
-      <c r="N19" s="65">
+      <c r="N19" s="62">
         <f t="shared" ref="N19" si="8">M19*K19</f>
         <v>1.6</v>
       </c>
@@ -2328,11 +2331,11 @@
     </row>
     <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="57">
+      <c r="B20" s="54">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="36" t="s">
@@ -2342,16 +2345,16 @@
         <v>72</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="G20" s="69" t="s">
-        <v>136</v>
+        <v>107</v>
+      </c>
+      <c r="G20" s="66" t="s">
+        <v>132</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J20" s="36">
         <v>1</v>
@@ -2360,22 +2363,22 @@
         <f>J20*5</f>
         <v>5</v>
       </c>
-      <c r="L20" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M20" s="64"/>
-      <c r="N20" s="64" t="s">
-        <v>218</v>
+      <c r="L20" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M20" s="61"/>
+      <c r="N20" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="O20" s="36"/>
     </row>
     <row r="21" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="59">
+      <c r="B21" s="56">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="60" t="s">
+      <c r="C21" s="57" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="38" t="s">
@@ -2385,16 +2388,16 @@
         <v>73</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="G21" s="70" t="s">
-        <v>137</v>
+        <v>108</v>
+      </c>
+      <c r="G21" s="67" t="s">
+        <v>133</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J21" s="38">
         <v>1</v>
@@ -2403,22 +2406,22 @@
         <f t="shared" ref="K21" si="9">J21*5</f>
         <v>5</v>
       </c>
-      <c r="L21" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M21" s="65"/>
-      <c r="N21" s="65" t="s">
-        <v>218</v>
+      <c r="L21" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M21" s="62"/>
+      <c r="N21" s="62" t="s">
+        <v>212</v>
       </c>
       <c r="O21" s="38"/>
     </row>
     <row r="22" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="57">
+      <c r="B22" s="54">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="58" t="s">
+      <c r="C22" s="55" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="36" t="s">
@@ -2428,16 +2431,16 @@
         <v>74</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>111</v>
-      </c>
-      <c r="G22" s="69" t="s">
-        <v>138</v>
+        <v>109</v>
+      </c>
+      <c r="G22" s="66" t="s">
+        <v>134</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J22" s="36">
         <v>1</v>
@@ -2446,22 +2449,22 @@
         <f>J22*5</f>
         <v>5</v>
       </c>
-      <c r="L22" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M22" s="64"/>
-      <c r="N22" s="64" t="s">
-        <v>218</v>
+      <c r="L22" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M22" s="61"/>
+      <c r="N22" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="O22" s="36"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="59">
+      <c r="B23" s="56">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="60" t="s">
+      <c r="C23" s="57" t="s">
         <v>10</v>
       </c>
       <c r="D23" s="38" t="s">
@@ -2471,16 +2474,16 @@
         <v>75</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>112</v>
-      </c>
-      <c r="G23" s="70" t="s">
-        <v>139</v>
+        <v>110</v>
+      </c>
+      <c r="G23" s="67" t="s">
+        <v>135</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J23" s="38">
         <v>2</v>
@@ -2489,13 +2492,13 @@
         <f t="shared" ref="K23" si="10">J23*5</f>
         <v>10</v>
       </c>
-      <c r="L23" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M23" s="65">
+      <c r="L23" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M23" s="62">
         <v>0.38</v>
       </c>
-      <c r="N23" s="65">
+      <c r="N23" s="62">
         <f t="shared" ref="N23" si="11">M23*K23</f>
         <v>3.8</v>
       </c>
@@ -2503,30 +2506,30 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="57">
+      <c r="B24" s="54">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="58" t="s">
-        <v>217</v>
-      </c>
-      <c r="D24" s="61" t="s">
+      <c r="C24" s="55" t="s">
+        <v>211</v>
+      </c>
+      <c r="D24" s="58" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="61" t="s">
+      <c r="E24" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="F24" s="62" t="s">
-        <v>216</v>
-      </c>
-      <c r="G24" s="61" t="s">
-        <v>113</v>
-      </c>
-      <c r="H24" s="61" t="s">
-        <v>218</v>
-      </c>
-      <c r="I24" s="61" t="s">
-        <v>218</v>
+      <c r="F24" s="59" t="s">
+        <v>210</v>
+      </c>
+      <c r="G24" s="58" t="s">
+        <v>111</v>
+      </c>
+      <c r="H24" s="58" t="s">
+        <v>212</v>
+      </c>
+      <c r="I24" s="58" t="s">
+        <v>212</v>
       </c>
       <c r="J24" s="36">
         <v>1</v>
@@ -2536,42 +2539,42 @@
         <v>5</v>
       </c>
       <c r="L24" s="36" t="s">
-        <v>218</v>
-      </c>
-      <c r="M24" s="66" t="s">
-        <v>218</v>
-      </c>
-      <c r="N24" s="66" t="s">
-        <v>218</v>
+        <v>212</v>
+      </c>
+      <c r="M24" s="63" t="s">
+        <v>212</v>
+      </c>
+      <c r="N24" s="63" t="s">
+        <v>212</v>
       </c>
       <c r="O24" s="36"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="59">
+      <c r="B25" s="56">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="60" t="s">
+      <c r="C25" s="57" t="s">
         <v>11</v>
       </c>
       <c r="D25" s="38" t="s">
         <v>34</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>77</v>
+        <v>225</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>216</v>
-      </c>
-      <c r="G25" s="70" t="s">
-        <v>114</v>
+        <v>210</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>226</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>176</v>
+        <v>227</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J25" s="38">
         <v>1</v>
@@ -2580,44 +2583,44 @@
         <f t="shared" ref="K25" si="12">J25*5</f>
         <v>5</v>
       </c>
-      <c r="L25" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M25" s="65">
-        <v>3.16</v>
-      </c>
-      <c r="N25" s="65">
+      <c r="L25" s="60" t="s">
+        <v>228</v>
+      </c>
+      <c r="M25" s="62">
+        <v>3.47</v>
+      </c>
+      <c r="N25" s="62">
         <f t="shared" ref="N25" si="13">M25*K25</f>
-        <v>15.8</v>
+        <v>17.350000000000001</v>
       </c>
       <c r="O25" s="38"/>
     </row>
     <row r="26" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="57">
+      <c r="B26" s="54">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="58" t="s">
+      <c r="C26" s="55" t="s">
         <v>12</v>
       </c>
       <c r="D26" s="36" t="s">
         <v>35</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F26" s="38" t="s">
-        <v>216</v>
-      </c>
-      <c r="G26" s="69" t="s">
-        <v>140</v>
+        <v>210</v>
+      </c>
+      <c r="G26" s="66" t="s">
+        <v>136</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="J26" s="36">
         <v>1</v>
@@ -2626,41 +2629,41 @@
         <f>J26*5</f>
         <v>5</v>
       </c>
-      <c r="L26" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M26" s="64"/>
-      <c r="N26" s="64" t="s">
-        <v>218</v>
+      <c r="L26" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M26" s="61"/>
+      <c r="N26" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="O26" s="36"/>
     </row>
     <row r="27" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="59">
+      <c r="B27" s="56">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="60" t="s">
+      <c r="C27" s="57" t="s">
         <v>13</v>
       </c>
       <c r="D27" s="38" t="s">
         <v>36</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>115</v>
-      </c>
-      <c r="G27" s="70" t="s">
-        <v>141</v>
+        <v>112</v>
+      </c>
+      <c r="G27" s="67" t="s">
+        <v>137</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J27" s="38">
         <v>1</v>
@@ -2669,41 +2672,41 @@
         <f t="shared" ref="K27" si="14">J27*5</f>
         <v>5</v>
       </c>
-      <c r="L27" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M27" s="65"/>
-      <c r="N27" s="65" t="s">
-        <v>218</v>
+      <c r="L27" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M27" s="62"/>
+      <c r="N27" s="62" t="s">
+        <v>212</v>
       </c>
       <c r="O27" s="38"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="57">
+      <c r="B28" s="54">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="60" t="s">
+      <c r="C28" s="57" t="s">
         <v>13</v>
       </c>
       <c r="D28" s="36" t="s">
         <v>37</v>
       </c>
       <c r="E28" s="36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>116</v>
-      </c>
-      <c r="G28" s="69" t="s">
-        <v>142</v>
+        <v>113</v>
+      </c>
+      <c r="G28" s="66" t="s">
+        <v>138</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="I28" s="38" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J28" s="36">
         <v>1</v>
@@ -2712,13 +2715,13 @@
         <f>J28*5</f>
         <v>5</v>
       </c>
-      <c r="L28" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M28" s="64">
+      <c r="L28" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M28" s="61">
         <v>0.46</v>
       </c>
-      <c r="N28" s="64">
+      <c r="N28" s="61">
         <f>M28*K28</f>
         <v>2.3000000000000003</v>
       </c>
@@ -2726,30 +2729,30 @@
     </row>
     <row r="29" spans="1:15" ht="36" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="59">
+      <c r="B29" s="56">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="60" t="s">
+      <c r="C29" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D29" s="38" t="s">
         <v>38</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>117</v>
-      </c>
-      <c r="G29" s="70" t="s">
-        <v>143</v>
+        <v>114</v>
+      </c>
+      <c r="G29" s="67" t="s">
+        <v>139</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="J29" s="38">
         <v>1</v>
@@ -2758,41 +2761,41 @@
         <f t="shared" ref="K29" si="15">J29*5</f>
         <v>5</v>
       </c>
-      <c r="L29" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M29" s="65"/>
-      <c r="N29" s="65" t="s">
-        <v>218</v>
+      <c r="L29" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M29" s="62"/>
+      <c r="N29" s="62" t="s">
+        <v>212</v>
       </c>
       <c r="O29" s="38"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="57">
+      <c r="B30" s="54">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="58" t="s">
+      <c r="C30" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D30" s="36" t="s">
         <v>39</v>
       </c>
       <c r="E30" s="36" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>117</v>
-      </c>
-      <c r="G30" s="69" t="s">
-        <v>144</v>
+        <v>114</v>
+      </c>
+      <c r="G30" s="66" t="s">
+        <v>140</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="J30" s="36">
         <v>1</v>
@@ -2801,13 +2804,13 @@
         <f>J30*5</f>
         <v>5</v>
       </c>
-      <c r="L30" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M30" s="64">
+      <c r="L30" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M30" s="61">
         <v>0.2155</v>
       </c>
-      <c r="N30" s="64">
+      <c r="N30" s="61">
         <f>M30*K30</f>
         <v>1.0774999999999999</v>
       </c>
@@ -2815,30 +2818,30 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="59">
+      <c r="B31" s="56">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="60" t="s">
+      <c r="C31" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D31" s="38" t="s">
         <v>40</v>
       </c>
       <c r="E31" s="38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>118</v>
-      </c>
-      <c r="G31" s="70" t="s">
-        <v>145</v>
+        <v>115</v>
+      </c>
+      <c r="G31" s="67" t="s">
+        <v>141</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I31" s="38" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="J31" s="38">
         <v>1</v>
@@ -2847,13 +2850,13 @@
         <f t="shared" ref="K31" si="16">J31*5</f>
         <v>5</v>
       </c>
-      <c r="L31" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M31" s="65">
+      <c r="L31" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M31" s="62">
         <v>0.1</v>
       </c>
-      <c r="N31" s="65">
+      <c r="N31" s="62">
         <f t="shared" ref="N31" si="17">M31*K31</f>
         <v>0.5</v>
       </c>
@@ -2861,30 +2864,30 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="57">
+      <c r="B32" s="54">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="58" t="s">
+      <c r="C32" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D32" s="36" t="s">
         <v>41</v>
       </c>
       <c r="E32" s="36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="G32" s="69" t="s">
-        <v>146</v>
+        <v>116</v>
+      </c>
+      <c r="G32" s="66" t="s">
+        <v>142</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="J32" s="36">
         <v>1</v>
@@ -2893,13 +2896,13 @@
         <f>J32*5</f>
         <v>5</v>
       </c>
-      <c r="L32" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M32" s="64">
+      <c r="L32" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M32" s="61">
         <v>0.9</v>
       </c>
-      <c r="N32" s="64">
+      <c r="N32" s="61">
         <f>M32*K32</f>
         <v>4.5</v>
       </c>
@@ -2907,30 +2910,30 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="59">
+      <c r="B33" s="56">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="60" t="s">
+      <c r="C33" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D33" s="38" t="s">
         <v>42</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>117</v>
-      </c>
-      <c r="G33" s="70" t="s">
-        <v>147</v>
+        <v>114</v>
+      </c>
+      <c r="G33" s="67" t="s">
+        <v>143</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J33" s="38">
         <v>1</v>
@@ -2939,13 +2942,13 @@
         <f t="shared" ref="K33" si="18">J33*5</f>
         <v>5</v>
       </c>
-      <c r="L33" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M33" s="65">
+      <c r="L33" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M33" s="62">
         <v>0.1</v>
       </c>
-      <c r="N33" s="65">
+      <c r="N33" s="62">
         <f t="shared" ref="N33" si="19">M33*K33</f>
         <v>0.5</v>
       </c>
@@ -2953,30 +2956,30 @@
     </row>
     <row r="34" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="57">
+      <c r="B34" s="54">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="58" t="s">
+      <c r="C34" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D34" s="36" t="s">
         <v>43</v>
       </c>
       <c r="E34" s="36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>117</v>
-      </c>
-      <c r="G34" s="69" t="s">
-        <v>148</v>
+        <v>114</v>
+      </c>
+      <c r="G34" s="66" t="s">
+        <v>144</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="J34" s="36">
         <v>1</v>
@@ -2985,41 +2988,41 @@
         <f>J34*5</f>
         <v>5</v>
       </c>
-      <c r="L34" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M34" s="64"/>
-      <c r="N34" s="64" t="s">
-        <v>218</v>
+      <c r="L34" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M34" s="61"/>
+      <c r="N34" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="O34" s="36"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="59">
+      <c r="B35" s="56">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="58" t="s">
+      <c r="C35" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D35" s="38" t="s">
         <v>44</v>
       </c>
       <c r="E35" s="38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="G35" s="69" t="s">
-        <v>149</v>
+        <v>117</v>
+      </c>
+      <c r="G35" s="66" t="s">
+        <v>145</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="I35" s="38" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="J35" s="38">
         <v>1</v>
@@ -3028,13 +3031,13 @@
         <f t="shared" ref="K35" si="20">J35*5</f>
         <v>5</v>
       </c>
-      <c r="L35" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M35" s="65">
+      <c r="L35" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M35" s="62">
         <v>0.15</v>
       </c>
-      <c r="N35" s="65">
+      <c r="N35" s="62">
         <f t="shared" ref="N35" si="21">M35*K35</f>
         <v>0.75</v>
       </c>
@@ -3042,30 +3045,30 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="57">
+      <c r="B36" s="54">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="58" t="s">
+      <c r="C36" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D36" s="36" t="s">
         <v>45</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>117</v>
-      </c>
-      <c r="G36" s="69" t="s">
-        <v>150</v>
+        <v>114</v>
+      </c>
+      <c r="G36" s="66" t="s">
+        <v>146</v>
       </c>
       <c r="H36" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="J36" s="36">
         <v>1</v>
@@ -3074,13 +3077,13 @@
         <f>J36*5</f>
         <v>5</v>
       </c>
-      <c r="L36" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M36" s="64">
+      <c r="L36" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M36" s="61">
         <v>0.1</v>
       </c>
-      <c r="N36" s="64">
+      <c r="N36" s="61">
         <f>M36*K36</f>
         <v>0.5</v>
       </c>
@@ -3088,30 +3091,30 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="59">
+      <c r="B37" s="56">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="60" t="s">
+      <c r="C37" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D37" s="38" t="s">
         <v>46</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F37" s="38" t="s">
-        <v>117</v>
-      </c>
-      <c r="G37" s="70" t="s">
-        <v>151</v>
+        <v>114</v>
+      </c>
+      <c r="G37" s="67" t="s">
+        <v>147</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="J37" s="38">
         <v>1</v>
@@ -3120,13 +3123,13 @@
         <f t="shared" ref="K37" si="22">J37*5</f>
         <v>5</v>
       </c>
-      <c r="L37" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M37" s="64">
+      <c r="L37" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M37" s="61">
         <v>0.1</v>
       </c>
-      <c r="N37" s="65">
+      <c r="N37" s="62">
         <f t="shared" ref="N37" si="23">M37*K37</f>
         <v>0.5</v>
       </c>
@@ -3134,30 +3137,30 @@
     </row>
     <row r="38" spans="1:15" ht="24" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="57">
+      <c r="B38" s="54">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="58" t="s">
+      <c r="C38" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D38" s="36" t="s">
         <v>47</v>
       </c>
       <c r="E38" s="36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>117</v>
-      </c>
-      <c r="G38" s="69" t="s">
-        <v>152</v>
+        <v>114</v>
+      </c>
+      <c r="G38" s="66" t="s">
+        <v>148</v>
       </c>
       <c r="H38" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="J38" s="36">
         <v>17</v>
@@ -3166,13 +3169,13 @@
         <f>J38*5</f>
         <v>85</v>
       </c>
-      <c r="L38" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M38" s="64">
+      <c r="L38" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M38" s="61">
         <v>1.6199999999999999E-2</v>
       </c>
-      <c r="N38" s="64">
+      <c r="N38" s="61">
         <f>M38*K38</f>
         <v>1.377</v>
       </c>
@@ -3180,30 +3183,30 @@
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="59">
+      <c r="B39" s="56">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="60" t="s">
+      <c r="C39" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D39" s="38" t="s">
         <v>48</v>
       </c>
       <c r="E39" s="38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="G39" s="70" t="s">
-        <v>153</v>
+        <v>117</v>
+      </c>
+      <c r="G39" s="67" t="s">
+        <v>149</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I39" s="38" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="J39" s="38">
         <v>1</v>
@@ -3212,13 +3215,13 @@
         <f t="shared" ref="K39" si="24">J39*5</f>
         <v>5</v>
       </c>
-      <c r="L39" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M39" s="65">
+      <c r="L39" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M39" s="62">
         <v>0.1</v>
       </c>
-      <c r="N39" s="65">
+      <c r="N39" s="62">
         <f t="shared" ref="N39" si="25">M39*K39</f>
         <v>0.5</v>
       </c>
@@ -3226,30 +3229,30 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="57">
+      <c r="B40" s="54">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
-      <c r="C40" s="58" t="s">
+      <c r="C40" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D40" s="36" t="s">
         <v>49</v>
       </c>
       <c r="E40" s="36" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="G40" s="69" t="s">
-        <v>154</v>
+        <v>117</v>
+      </c>
+      <c r="G40" s="66" t="s">
+        <v>150</v>
       </c>
       <c r="H40" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="J40" s="36">
         <v>2</v>
@@ -3258,13 +3261,13 @@
         <f>J40*5</f>
         <v>10</v>
       </c>
-      <c r="L40" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M40" s="64">
+      <c r="L40" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M40" s="61">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="N40" s="64">
+      <c r="N40" s="61">
         <f>M40*K40</f>
         <v>0.15</v>
       </c>
@@ -3272,30 +3275,30 @@
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="59">
+      <c r="B41" s="56">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="60" t="s">
+      <c r="C41" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D41" s="38" t="s">
         <v>50</v>
       </c>
       <c r="E41" s="38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F41" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="G41" s="70" t="s">
-        <v>155</v>
+        <v>117</v>
+      </c>
+      <c r="G41" s="67" t="s">
+        <v>151</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I41" s="38" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="J41" s="38">
         <v>2</v>
@@ -3304,13 +3307,13 @@
         <f t="shared" ref="K41" si="26">J41*5</f>
         <v>10</v>
       </c>
-      <c r="L41" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M41" s="65">
+      <c r="L41" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M41" s="62">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="N41" s="65">
+      <c r="N41" s="62">
         <f t="shared" ref="N41" si="27">M41*K41</f>
         <v>0.18</v>
       </c>
@@ -3318,30 +3321,30 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="57">
+      <c r="B42" s="54">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="58" t="s">
+      <c r="C42" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D42" s="36" t="s">
         <v>51</v>
       </c>
       <c r="E42" s="36" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>117</v>
-      </c>
-      <c r="G42" s="69" t="s">
-        <v>156</v>
+        <v>114</v>
+      </c>
+      <c r="G42" s="66" t="s">
+        <v>152</v>
       </c>
       <c r="H42" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="J42" s="36">
         <v>4</v>
@@ -3350,13 +3353,13 @@
         <f>J42*5</f>
         <v>20</v>
       </c>
-      <c r="L42" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M42" s="64">
+      <c r="L42" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M42" s="61">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="N42" s="64">
+      <c r="N42" s="61">
         <f>M42*K42</f>
         <v>0.52</v>
       </c>
@@ -3364,30 +3367,30 @@
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
-      <c r="B43" s="59">
+      <c r="B43" s="56">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="60" t="s">
+      <c r="C43" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D43" s="38" t="s">
         <v>52</v>
       </c>
       <c r="E43" s="38" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F43" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="G43" s="70" t="s">
-        <v>157</v>
+        <v>117</v>
+      </c>
+      <c r="G43" s="67" t="s">
+        <v>153</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I43" s="38" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="J43" s="38">
         <v>1</v>
@@ -3396,13 +3399,13 @@
         <f t="shared" ref="K43" si="28">J43*5</f>
         <v>5</v>
       </c>
-      <c r="L43" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M43" s="65">
+      <c r="L43" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M43" s="62">
         <v>0.1</v>
       </c>
-      <c r="N43" s="65">
+      <c r="N43" s="62">
         <f t="shared" ref="N43" si="29">M43*K43</f>
         <v>0.5</v>
       </c>
@@ -3410,30 +3413,30 @@
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="57">
+      <c r="B44" s="54">
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
-      <c r="C44" s="58" t="s">
+      <c r="C44" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D44" s="36" t="s">
         <v>53</v>
       </c>
       <c r="E44" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="G44" s="69" t="s">
-        <v>158</v>
+        <v>117</v>
+      </c>
+      <c r="G44" s="66" t="s">
+        <v>154</v>
       </c>
       <c r="H44" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="J44" s="36">
         <v>4</v>
@@ -3442,13 +3445,13 @@
         <f>J44*5</f>
         <v>20</v>
       </c>
-      <c r="L44" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M44" s="64">
+      <c r="L44" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M44" s="61">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="N44" s="64">
+      <c r="N44" s="61">
         <f>M44*K44</f>
         <v>0.36</v>
       </c>
@@ -3456,30 +3459,30 @@
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
-      <c r="B45" s="59">
+      <c r="B45" s="56">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="58" t="s">
+      <c r="C45" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D45" s="38" t="s">
         <v>54</v>
       </c>
       <c r="E45" s="38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F45" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="G45" s="70" t="s">
-        <v>159</v>
+        <v>117</v>
+      </c>
+      <c r="G45" s="67" t="s">
+        <v>155</v>
       </c>
       <c r="H45" s="38" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I45" s="38" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="J45" s="38">
         <v>1</v>
@@ -3488,13 +3491,13 @@
         <f t="shared" ref="K45" si="30">J45*5</f>
         <v>5</v>
       </c>
-      <c r="L45" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M45" s="65">
+      <c r="L45" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M45" s="62">
         <v>0.1</v>
       </c>
-      <c r="N45" s="65">
+      <c r="N45" s="62">
         <f t="shared" ref="N45" si="31">M45*K45</f>
         <v>0.5</v>
       </c>
@@ -3502,30 +3505,30 @@
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="57">
+      <c r="B46" s="54">
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="58" t="s">
+      <c r="C46" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D46" s="36" t="s">
         <v>55</v>
       </c>
       <c r="E46" s="36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="G46" s="69" t="s">
-        <v>160</v>
+        <v>117</v>
+      </c>
+      <c r="G46" s="66" t="s">
+        <v>156</v>
       </c>
       <c r="H46" s="36" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I46" s="36" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="J46" s="36">
         <v>1</v>
@@ -3534,13 +3537,13 @@
         <f>J46*5</f>
         <v>5</v>
       </c>
-      <c r="L46" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M46" s="64">
+      <c r="L46" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M46" s="61">
         <v>0.1</v>
       </c>
-      <c r="N46" s="64">
+      <c r="N46" s="61">
         <f>M46*K46</f>
         <v>0.5</v>
       </c>
@@ -3548,30 +3551,30 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="59">
+      <c r="B47" s="56">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="60" t="s">
+      <c r="C47" s="57" t="s">
         <v>15</v>
       </c>
       <c r="D47" s="38" t="s">
         <v>56</v>
       </c>
       <c r="E47" s="38" t="s">
-        <v>99</v>
+        <v>229</v>
       </c>
       <c r="F47" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="G47" s="70" t="s">
-        <v>161</v>
+        <v>230</v>
+      </c>
+      <c r="G47" s="38" t="s">
+        <v>231</v>
       </c>
       <c r="H47" s="38" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="I47" s="38" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J47" s="38">
         <v>1</v>
@@ -3580,42 +3583,44 @@
         <f t="shared" ref="K47" si="32">J47*5</f>
         <v>5</v>
       </c>
-      <c r="L47" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="M47" s="65"/>
-      <c r="N47" s="65">
+      <c r="L47" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M47" s="62">
+        <v>2.97</v>
+      </c>
+      <c r="N47" s="62">
         <f t="shared" ref="N47" si="33">M47*K47</f>
-        <v>0</v>
+        <v>14.850000000000001</v>
       </c>
       <c r="O47" s="38"/>
     </row>
     <row r="48" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
-      <c r="B48" s="57">
+      <c r="B48" s="54">
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
-      <c r="C48" s="58" t="s">
+      <c r="C48" s="55" t="s">
         <v>15</v>
       </c>
       <c r="D48" s="36" t="s">
         <v>57</v>
       </c>
       <c r="E48" s="36" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="G48" s="69" t="s">
-        <v>162</v>
+        <v>118</v>
+      </c>
+      <c r="G48" s="66" t="s">
+        <v>157</v>
       </c>
       <c r="H48" s="36" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J48" s="36">
         <v>1</v>
@@ -3624,41 +3629,41 @@
         <f>J48*5</f>
         <v>5</v>
       </c>
-      <c r="L48" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M48" s="64"/>
-      <c r="N48" s="64" t="s">
-        <v>218</v>
+      <c r="L48" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M48" s="61"/>
+      <c r="N48" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="O48" s="36"/>
     </row>
     <row r="49" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
-      <c r="B49" s="59">
+      <c r="B49" s="56">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C49" s="60" t="s">
+      <c r="C49" s="57" t="s">
         <v>15</v>
       </c>
       <c r="D49" s="38" t="s">
         <v>58</v>
       </c>
       <c r="E49" s="38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F49" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="G49" s="70" t="s">
-        <v>163</v>
+        <v>119</v>
+      </c>
+      <c r="G49" s="67" t="s">
+        <v>158</v>
       </c>
       <c r="H49" s="38" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="I49" s="38" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J49" s="38">
         <v>1</v>
@@ -3667,41 +3672,41 @@
         <f t="shared" ref="K49" si="34">J49*5</f>
         <v>5</v>
       </c>
-      <c r="L49" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M49" s="65"/>
-      <c r="N49" s="65" t="s">
-        <v>218</v>
+      <c r="L49" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M49" s="62"/>
+      <c r="N49" s="62" t="s">
+        <v>212</v>
       </c>
       <c r="O49" s="38"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
-      <c r="B50" s="57">
+      <c r="B50" s="54">
         <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
-      <c r="C50" s="58" t="s">
+      <c r="C50" s="55" t="s">
         <v>16</v>
       </c>
       <c r="D50" s="36" t="s">
         <v>59</v>
       </c>
       <c r="E50" s="36" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>124</v>
-      </c>
-      <c r="G50" s="69" t="s">
-        <v>164</v>
+        <v>120</v>
+      </c>
+      <c r="G50" s="66" t="s">
+        <v>159</v>
       </c>
       <c r="H50" s="36" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I50" s="36" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J50" s="36">
         <v>1</v>
@@ -3710,13 +3715,13 @@
         <f>J50*5</f>
         <v>5</v>
       </c>
-      <c r="L50" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="M50" s="64">
+      <c r="L50" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="M50" s="61">
         <v>0.87</v>
       </c>
-      <c r="N50" s="64">
+      <c r="N50" s="61">
         <f>M50*K50</f>
         <v>4.3499999999999996</v>
       </c>
@@ -3724,30 +3729,30 @@
     </row>
     <row r="51" spans="1:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
-      <c r="B51" s="59">
+      <c r="B51" s="56">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="60" t="s">
+      <c r="C51" s="57" t="s">
         <v>17</v>
       </c>
       <c r="D51" s="38" t="s">
         <v>60</v>
       </c>
       <c r="E51" s="38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F51" s="38" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G51" s="38" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="H51" s="38" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="I51" s="36" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J51" s="38">
         <v>1</v>
@@ -3756,12 +3761,12 @@
         <f t="shared" ref="K51" si="35">J51*5</f>
         <v>5</v>
       </c>
-      <c r="L51" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="M51" s="65"/>
-      <c r="N51" s="65" t="s">
-        <v>218</v>
+      <c r="L51" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="M51" s="62"/>
+      <c r="N51" s="62" t="s">
+        <v>212</v>
       </c>
       <c r="O51" s="38"/>
     </row>
@@ -3779,9 +3784,9 @@
       <c r="K52" s="35"/>
       <c r="L52" s="35"/>
       <c r="M52" s="35"/>
-      <c r="N52" s="67">
+      <c r="N52" s="64">
         <f>SUM(N10:N51)</f>
-        <v>60.154500000000006</v>
+        <v>76.55449999999999</v>
       </c>
       <c r="O52" s="41"/>
     </row>
@@ -3799,9 +3804,9 @@
       <c r="K53" s="9"/>
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
-      <c r="N53" s="68">
+      <c r="N53" s="65">
         <f>N52/5</f>
-        <v>12.030900000000001</v>
+        <v>15.310899999999998</v>
       </c>
       <c r="O53" s="42"/>
     </row>
@@ -3820,28 +3825,29 @@
     <hyperlink ref="L18" r:id="rId7"/>
     <hyperlink ref="L19" r:id="rId8"/>
     <hyperlink ref="L23" r:id="rId9"/>
-    <hyperlink ref="L25" r:id="rId10"/>
-    <hyperlink ref="L28" r:id="rId11"/>
-    <hyperlink ref="L30" r:id="rId12"/>
-    <hyperlink ref="L31" r:id="rId13"/>
-    <hyperlink ref="L32" r:id="rId14"/>
-    <hyperlink ref="L33" r:id="rId15"/>
-    <hyperlink ref="L35" r:id="rId16"/>
-    <hyperlink ref="L36" r:id="rId17"/>
-    <hyperlink ref="L37" r:id="rId18"/>
-    <hyperlink ref="L38" r:id="rId19"/>
-    <hyperlink ref="L39" r:id="rId20"/>
-    <hyperlink ref="L40" r:id="rId21"/>
-    <hyperlink ref="L41" r:id="rId22"/>
-    <hyperlink ref="L42" r:id="rId23"/>
-    <hyperlink ref="L43" r:id="rId24"/>
-    <hyperlink ref="L44" r:id="rId25"/>
-    <hyperlink ref="L45" r:id="rId26"/>
-    <hyperlink ref="L46" r:id="rId27"/>
-    <hyperlink ref="L50" r:id="rId28"/>
+    <hyperlink ref="L28" r:id="rId10"/>
+    <hyperlink ref="L30" r:id="rId11"/>
+    <hyperlink ref="L31" r:id="rId12"/>
+    <hyperlink ref="L32" r:id="rId13"/>
+    <hyperlink ref="L33" r:id="rId14"/>
+    <hyperlink ref="L35" r:id="rId15"/>
+    <hyperlink ref="L36" r:id="rId16"/>
+    <hyperlink ref="L37" r:id="rId17"/>
+    <hyperlink ref="L38" r:id="rId18"/>
+    <hyperlink ref="L39" r:id="rId19"/>
+    <hyperlink ref="L40" r:id="rId20"/>
+    <hyperlink ref="L41" r:id="rId21"/>
+    <hyperlink ref="L42" r:id="rId22"/>
+    <hyperlink ref="L43" r:id="rId23"/>
+    <hyperlink ref="L44" r:id="rId24"/>
+    <hyperlink ref="L45" r:id="rId25"/>
+    <hyperlink ref="L46" r:id="rId26"/>
+    <hyperlink ref="L50" r:id="rId27"/>
+    <hyperlink ref="L25" r:id="rId28"/>
+    <hyperlink ref="L47" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId29"/>
-  <drawing r:id="rId30"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#18 0R resistor Added 10K resistor remove
</commit_message>
<xml_diff>
--- a/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
+++ b/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
@@ -162,18 +162,12 @@
     <t>R9</t>
   </si>
   <si>
-    <t>R10, R11, R12, R14, R23, R25, R29, R30, R31, R34, R35, R36, R37, R38, R39, R41, R42</t>
-  </si>
-  <si>
     <t>R13</t>
   </si>
   <si>
     <t>R15, R16</t>
   </si>
   <si>
-    <t>R17, R33</t>
-  </si>
-  <si>
     <t>R18, R19, R27, R28</t>
   </si>
   <si>
@@ -715,6 +709,12 @@
   </si>
   <si>
     <t>TPS2375DR</t>
+  </si>
+  <si>
+    <t>R10, R14, R23, R25, R29, R30, R31, R34, R35, R36, R37, R38, R39</t>
+  </si>
+  <si>
+    <t>R12, R17, R33</t>
   </si>
 </sst>
 </file>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="50" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="51" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="52" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1838,37 +1838,37 @@
         <v>18</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I9" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>212</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>215</v>
+      </c>
+      <c r="N9" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="O9" s="29" t="s">
         <v>213</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>220</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>214</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>216</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>217</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1884,19 +1884,19 @@
         <v>19</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="J10" s="36">
         <v>10</v>
@@ -1906,7 +1906,7 @@
         <v>50</v>
       </c>
       <c r="L10" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M10" s="61">
         <v>1.26E-2</v>
@@ -1930,19 +1930,19 @@
         <v>20</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J11" s="38">
         <v>1</v>
@@ -1952,13 +1952,13 @@
         <v>5</v>
       </c>
       <c r="L11" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M11" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="N11" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O11" s="38"/>
     </row>
@@ -1975,19 +1975,19 @@
         <v>21</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G12" s="66" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="J12" s="36">
         <v>3</v>
@@ -1997,7 +1997,7 @@
         <v>15</v>
       </c>
       <c r="L12" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M12" s="61">
         <v>7.0999999999999994E-2</v>
@@ -2021,19 +2021,19 @@
         <v>22</v>
       </c>
       <c r="E13" s="38" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G13" s="67" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="J13" s="38">
         <v>1</v>
@@ -2043,7 +2043,7 @@
         <v>5</v>
       </c>
       <c r="L13" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M13" s="62">
         <v>2.33</v>
@@ -2067,19 +2067,19 @@
         <v>23</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G14" s="66" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="J14" s="36">
         <v>1</v>
@@ -2089,7 +2089,7 @@
         <v>5</v>
       </c>
       <c r="L14" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M14" s="61">
         <v>0.1</v>
@@ -2113,19 +2113,19 @@
         <v>24</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G15" s="66" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="J15" s="38">
         <v>3</v>
@@ -2135,7 +2135,7 @@
         <v>15</v>
       </c>
       <c r="L15" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M15" s="62">
         <v>5.5E-2</v>
@@ -2159,19 +2159,19 @@
         <v>25</v>
       </c>
       <c r="E16" s="36" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G16" s="66" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="J16" s="36">
         <v>1</v>
@@ -2181,7 +2181,7 @@
         <v>5</v>
       </c>
       <c r="L16" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M16" s="61">
         <v>0.75</v>
@@ -2205,19 +2205,19 @@
         <v>26</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G17" s="67" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="J17" s="38">
         <v>2</v>
@@ -2227,13 +2227,13 @@
         <v>10</v>
       </c>
       <c r="L17" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M17" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="N17" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O17" s="38"/>
     </row>
@@ -2250,19 +2250,19 @@
         <v>27</v>
       </c>
       <c r="E18" s="36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G18" s="66" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="J18" s="36">
         <v>2</v>
@@ -2272,7 +2272,7 @@
         <v>10</v>
       </c>
       <c r="L18" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M18" s="61">
         <v>9.7000000000000003E-2</v>
@@ -2296,19 +2296,19 @@
         <v>28</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G19" s="67" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="J19" s="38">
         <v>1</v>
@@ -2318,7 +2318,7 @@
         <v>5</v>
       </c>
       <c r="L19" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M19" s="62">
         <v>0.32</v>
@@ -2342,19 +2342,19 @@
         <v>29</v>
       </c>
       <c r="E20" s="36" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G20" s="66" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J20" s="36">
         <v>1</v>
@@ -2364,11 +2364,11 @@
         <v>5</v>
       </c>
       <c r="L20" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M20" s="61"/>
       <c r="N20" s="61" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O20" s="36"/>
     </row>
@@ -2385,19 +2385,19 @@
         <v>30</v>
       </c>
       <c r="E21" s="38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G21" s="67" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J21" s="38">
         <v>1</v>
@@ -2407,11 +2407,11 @@
         <v>5</v>
       </c>
       <c r="L21" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M21" s="62"/>
       <c r="N21" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O21" s="38"/>
     </row>
@@ -2428,19 +2428,19 @@
         <v>31</v>
       </c>
       <c r="E22" s="36" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G22" s="66" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J22" s="36">
         <v>1</v>
@@ -2450,11 +2450,11 @@
         <v>5</v>
       </c>
       <c r="L22" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M22" s="61"/>
       <c r="N22" s="61" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O22" s="36"/>
     </row>
@@ -2471,19 +2471,19 @@
         <v>32</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G23" s="67" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J23" s="38">
         <v>2</v>
@@ -2493,7 +2493,7 @@
         <v>10</v>
       </c>
       <c r="L23" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M23" s="62">
         <v>0.38</v>
@@ -2511,25 +2511,25 @@
         <v>15</v>
       </c>
       <c r="C24" s="55" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D24" s="58" t="s">
         <v>33</v>
       </c>
       <c r="E24" s="58" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F24" s="59" t="s">
+        <v>208</v>
+      </c>
+      <c r="G24" s="58" t="s">
+        <v>109</v>
+      </c>
+      <c r="H24" s="58" t="s">
         <v>210</v>
       </c>
-      <c r="G24" s="58" t="s">
-        <v>111</v>
-      </c>
-      <c r="H24" s="58" t="s">
-        <v>212</v>
-      </c>
       <c r="I24" s="58" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J24" s="36">
         <v>1</v>
@@ -2539,13 +2539,13 @@
         <v>5</v>
       </c>
       <c r="L24" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="M24" s="63" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="N24" s="63" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O24" s="36"/>
     </row>
@@ -2562,19 +2562,19 @@
         <v>34</v>
       </c>
       <c r="E25" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="F25" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>224</v>
+      </c>
+      <c r="H25" s="38" t="s">
         <v>225</v>
       </c>
-      <c r="F25" s="38" t="s">
+      <c r="I25" s="38" t="s">
         <v>210</v>
-      </c>
-      <c r="G25" s="38" t="s">
-        <v>226</v>
-      </c>
-      <c r="H25" s="38" t="s">
-        <v>227</v>
-      </c>
-      <c r="I25" s="38" t="s">
-        <v>212</v>
       </c>
       <c r="J25" s="38">
         <v>1</v>
@@ -2584,7 +2584,7 @@
         <v>5</v>
       </c>
       <c r="L25" s="60" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="M25" s="62">
         <v>3.47</v>
@@ -2608,19 +2608,19 @@
         <v>35</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F26" s="38" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="G26" s="66" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="J26" s="36">
         <v>1</v>
@@ -2630,11 +2630,11 @@
         <v>5</v>
       </c>
       <c r="L26" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M26" s="61"/>
       <c r="N26" s="61" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O26" s="36"/>
     </row>
@@ -2651,19 +2651,19 @@
         <v>36</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G27" s="67" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J27" s="38">
         <v>1</v>
@@ -2673,11 +2673,11 @@
         <v>5</v>
       </c>
       <c r="L27" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M27" s="62"/>
       <c r="N27" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O27" s="38"/>
     </row>
@@ -2694,19 +2694,19 @@
         <v>37</v>
       </c>
       <c r="E28" s="36" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G28" s="66" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I28" s="38" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J28" s="36">
         <v>1</v>
@@ -2716,7 +2716,7 @@
         <v>5</v>
       </c>
       <c r="L28" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M28" s="61">
         <v>0.46</v>
@@ -2740,19 +2740,19 @@
         <v>38</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G29" s="67" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J29" s="38">
         <v>1</v>
@@ -2762,11 +2762,11 @@
         <v>5</v>
       </c>
       <c r="L29" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M29" s="62"/>
       <c r="N29" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O29" s="38"/>
     </row>
@@ -2783,19 +2783,19 @@
         <v>39</v>
       </c>
       <c r="E30" s="36" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G30" s="66" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="J30" s="36">
         <v>1</v>
@@ -2805,7 +2805,7 @@
         <v>5</v>
       </c>
       <c r="L30" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M30" s="61">
         <v>0.2155</v>
@@ -2829,19 +2829,19 @@
         <v>40</v>
       </c>
       <c r="E31" s="38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G31" s="67" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I31" s="38" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J31" s="38">
         <v>1</v>
@@ -2851,7 +2851,7 @@
         <v>5</v>
       </c>
       <c r="L31" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M31" s="62">
         <v>0.1</v>
@@ -2875,19 +2875,19 @@
         <v>41</v>
       </c>
       <c r="E32" s="36" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G32" s="66" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="J32" s="36">
         <v>1</v>
@@ -2897,7 +2897,7 @@
         <v>5</v>
       </c>
       <c r="L32" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M32" s="61">
         <v>0.9</v>
@@ -2921,19 +2921,19 @@
         <v>42</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G33" s="67" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="J33" s="38">
         <v>1</v>
@@ -2943,7 +2943,7 @@
         <v>5</v>
       </c>
       <c r="L33" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M33" s="62">
         <v>0.1</v>
@@ -2967,19 +2967,19 @@
         <v>43</v>
       </c>
       <c r="E34" s="36" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G34" s="66" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J34" s="36">
         <v>1</v>
@@ -2989,11 +2989,11 @@
         <v>5</v>
       </c>
       <c r="L34" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M34" s="61"/>
       <c r="N34" s="61" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O34" s="36"/>
     </row>
@@ -3010,19 +3010,19 @@
         <v>44</v>
       </c>
       <c r="E35" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G35" s="66" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="I35" s="38" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="J35" s="38">
         <v>1</v>
@@ -3032,7 +3032,7 @@
         <v>5</v>
       </c>
       <c r="L35" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M35" s="62">
         <v>0.15</v>
@@ -3056,19 +3056,19 @@
         <v>45</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G36" s="66" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H36" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="J36" s="36">
         <v>1</v>
@@ -3078,7 +3078,7 @@
         <v>5</v>
       </c>
       <c r="L36" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M36" s="61">
         <v>0.1</v>
@@ -3102,19 +3102,19 @@
         <v>46</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F37" s="38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G37" s="67" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J37" s="38">
         <v>1</v>
@@ -3124,7 +3124,7 @@
         <v>5</v>
       </c>
       <c r="L37" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M37" s="61">
         <v>0.1</v>
@@ -3145,39 +3145,39 @@
         <v>14</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>47</v>
+        <v>230</v>
       </c>
       <c r="E38" s="36" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G38" s="66" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H38" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="J38" s="36">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K38" s="37">
         <f>J38*5</f>
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="L38" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M38" s="61">
         <v>1.6199999999999999E-2</v>
       </c>
       <c r="N38" s="61">
         <f>M38*K38</f>
-        <v>1.377</v>
+        <v>1.0529999999999999</v>
       </c>
       <c r="O38" s="36"/>
     </row>
@@ -3191,22 +3191,22 @@
         <v>14</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E39" s="38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G39" s="67" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I39" s="38" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="J39" s="38">
         <v>1</v>
@@ -3216,7 +3216,7 @@
         <v>5</v>
       </c>
       <c r="L39" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M39" s="62">
         <v>0.1</v>
@@ -3237,22 +3237,22 @@
         <v>14</v>
       </c>
       <c r="D40" s="36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E40" s="36" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G40" s="66" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H40" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="J40" s="36">
         <v>2</v>
@@ -3262,7 +3262,7 @@
         <v>10</v>
       </c>
       <c r="L40" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M40" s="61">
         <v>1.4999999999999999E-2</v>
@@ -3283,39 +3283,39 @@
         <v>14</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>50</v>
+        <v>231</v>
       </c>
       <c r="E41" s="38" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F41" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G41" s="67" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I41" s="38" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="J41" s="38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K41" s="39">
         <f t="shared" ref="K41" si="26">J41*5</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L41" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M41" s="62">
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="N41" s="62">
         <f t="shared" ref="N41" si="27">M41*K41</f>
-        <v>0.18</v>
+        <v>0.26999999999999996</v>
       </c>
       <c r="O41" s="38"/>
     </row>
@@ -3329,22 +3329,22 @@
         <v>14</v>
       </c>
       <c r="D42" s="36" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E42" s="36" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G42" s="66" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H42" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J42" s="36">
         <v>4</v>
@@ -3354,7 +3354,7 @@
         <v>20</v>
       </c>
       <c r="L42" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M42" s="61">
         <v>2.5999999999999999E-2</v>
@@ -3375,22 +3375,22 @@
         <v>14</v>
       </c>
       <c r="D43" s="38" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E43" s="38" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F43" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G43" s="67" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I43" s="38" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="J43" s="38">
         <v>1</v>
@@ -3400,7 +3400,7 @@
         <v>5</v>
       </c>
       <c r="L43" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M43" s="62">
         <v>0.1</v>
@@ -3421,22 +3421,22 @@
         <v>14</v>
       </c>
       <c r="D44" s="36" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E44" s="36" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G44" s="66" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H44" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="J44" s="36">
         <v>4</v>
@@ -3446,7 +3446,7 @@
         <v>20</v>
       </c>
       <c r="L44" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M44" s="61">
         <v>1.7999999999999999E-2</v>
@@ -3467,22 +3467,22 @@
         <v>14</v>
       </c>
       <c r="D45" s="38" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E45" s="38" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F45" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G45" s="67" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H45" s="38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I45" s="38" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="J45" s="38">
         <v>1</v>
@@ -3492,7 +3492,7 @@
         <v>5</v>
       </c>
       <c r="L45" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M45" s="62">
         <v>0.1</v>
@@ -3513,22 +3513,22 @@
         <v>14</v>
       </c>
       <c r="D46" s="36" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E46" s="36" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G46" s="66" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H46" s="36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I46" s="36" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J46" s="36">
         <v>1</v>
@@ -3538,7 +3538,7 @@
         <v>5</v>
       </c>
       <c r="L46" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M46" s="61">
         <v>0.1</v>
@@ -3559,22 +3559,22 @@
         <v>15</v>
       </c>
       <c r="D47" s="38" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E47" s="38" t="s">
+        <v>227</v>
+      </c>
+      <c r="F47" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="G47" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="F47" s="38" t="s">
-        <v>230</v>
-      </c>
-      <c r="G47" s="38" t="s">
-        <v>231</v>
-      </c>
       <c r="H47" s="38" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="I47" s="38" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J47" s="38">
         <v>1</v>
@@ -3584,7 +3584,7 @@
         <v>5</v>
       </c>
       <c r="L47" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M47" s="62">
         <v>2.97</v>
@@ -3605,22 +3605,22 @@
         <v>15</v>
       </c>
       <c r="D48" s="36" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E48" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G48" s="66" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H48" s="36" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J48" s="36">
         <v>1</v>
@@ -3630,11 +3630,11 @@
         <v>5</v>
       </c>
       <c r="L48" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M48" s="61"/>
       <c r="N48" s="61" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O48" s="36"/>
     </row>
@@ -3648,22 +3648,22 @@
         <v>15</v>
       </c>
       <c r="D49" s="38" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E49" s="38" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F49" s="38" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G49" s="67" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H49" s="38" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I49" s="38" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J49" s="38">
         <v>1</v>
@@ -3673,11 +3673,11 @@
         <v>5</v>
       </c>
       <c r="L49" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M49" s="62"/>
       <c r="N49" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O49" s="38"/>
     </row>
@@ -3691,22 +3691,22 @@
         <v>16</v>
       </c>
       <c r="D50" s="36" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E50" s="36" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G50" s="66" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H50" s="36" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="I50" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J50" s="36">
         <v>1</v>
@@ -3716,7 +3716,7 @@
         <v>5</v>
       </c>
       <c r="L50" s="60" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M50" s="61">
         <v>0.87</v>
@@ -3737,22 +3737,22 @@
         <v>17</v>
       </c>
       <c r="D51" s="38" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E51" s="38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F51" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="G51" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="H51" s="38" t="s">
+        <v>178</v>
+      </c>
+      <c r="I51" s="36" t="s">
         <v>210</v>
-      </c>
-      <c r="G51" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="H51" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="I51" s="36" t="s">
-        <v>212</v>
       </c>
       <c r="J51" s="38">
         <v>1</v>
@@ -3762,11 +3762,11 @@
         <v>5</v>
       </c>
       <c r="L51" s="60" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M51" s="62"/>
       <c r="N51" s="62" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O51" s="38"/>
     </row>
@@ -3786,7 +3786,7 @@
       <c r="M52" s="35"/>
       <c r="N52" s="64">
         <f>SUM(N10:N51)</f>
-        <v>76.55449999999999</v>
+        <v>76.320499999999996</v>
       </c>
       <c r="O52" s="41"/>
     </row>
@@ -3806,7 +3806,7 @@
       <c r="M53" s="9"/>
       <c r="N53" s="65">
         <f>N52/5</f>
-        <v>15.310899999999998</v>
+        <v>15.264099999999999</v>
       </c>
       <c r="O53" s="42"/>
     </row>

</xml_diff>

<commit_message>
#18 Fuse and R11 added in BOM
</commit_message>
<xml_diff>
--- a/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
+++ b/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
@@ -141,9 +141,6 @@
     <t>R2</t>
   </si>
   <si>
-    <t>R3</t>
-  </si>
-  <si>
     <t>R4</t>
   </si>
   <si>
@@ -237,9 +234,6 @@
     <t>SCHOTTKY DIODE SMB 100V 5A</t>
   </si>
   <si>
-    <t>6V 1A 100A 1.95A - Resettable Fuses ROHS</t>
-  </si>
-  <si>
     <t>FERRITE BEAD 600 OHM 1210 1LN</t>
   </si>
   <si>
@@ -417,9 +411,6 @@
     <t>SS510B</t>
   </si>
   <si>
-    <t>JK-SMD0805-100-6</t>
-  </si>
-  <si>
     <t>FBMH3225HM601NT</t>
   </si>
   <si>
@@ -522,9 +513,6 @@
     <t>MDD</t>
   </si>
   <si>
-    <t>Jinrui Electronic Materials Co.</t>
-  </si>
-  <si>
     <t>Taiyo Yuden</t>
   </si>
   <si>
@@ -715,6 +703,18 @@
   </si>
   <si>
     <t>R12, R17, R33</t>
+  </si>
+  <si>
+    <t>6V 2A 50A 1W -40℃~+85℃ 4A 4mΩ 5s 45mΩ 0805 Resettable Fuses ROHS</t>
+  </si>
+  <si>
+    <t>BSMD0805L-200</t>
+  </si>
+  <si>
+    <t>BHFUSE</t>
+  </si>
+  <si>
+    <t>R3, R11</t>
   </si>
 </sst>
 </file>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="50" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="51" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="52" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1838,37 +1838,37 @@
         <v>18</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I9" s="30" t="s">
+        <v>207</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="J9" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="K9" s="29" t="s">
+      <c r="N9" s="29" t="s">
         <v>212</v>
       </c>
-      <c r="L9" s="29" t="s">
-        <v>214</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>215</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>216</v>
-      </c>
       <c r="O9" s="29" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1884,19 +1884,19 @@
         <v>19</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="J10" s="36">
         <v>10</v>
@@ -1906,7 +1906,7 @@
         <v>50</v>
       </c>
       <c r="L10" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M10" s="61">
         <v>1.26E-2</v>
@@ -1930,19 +1930,19 @@
         <v>20</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="J11" s="38">
         <v>1</v>
@@ -1952,13 +1952,13 @@
         <v>5</v>
       </c>
       <c r="L11" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M11" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="N11" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O11" s="38"/>
     </row>
@@ -1975,19 +1975,19 @@
         <v>21</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G12" s="66" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="J12" s="36">
         <v>3</v>
@@ -1997,7 +1997,7 @@
         <v>15</v>
       </c>
       <c r="L12" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M12" s="61">
         <v>7.0999999999999994E-2</v>
@@ -2021,19 +2021,19 @@
         <v>22</v>
       </c>
       <c r="E13" s="38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G13" s="67" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J13" s="38">
         <v>1</v>
@@ -2043,7 +2043,7 @@
         <v>5</v>
       </c>
       <c r="L13" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M13" s="62">
         <v>2.33</v>
@@ -2067,19 +2067,19 @@
         <v>23</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G14" s="66" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="J14" s="36">
         <v>1</v>
@@ -2089,7 +2089,7 @@
         <v>5</v>
       </c>
       <c r="L14" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M14" s="61">
         <v>0.1</v>
@@ -2113,19 +2113,19 @@
         <v>24</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G15" s="66" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J15" s="38">
         <v>3</v>
@@ -2135,7 +2135,7 @@
         <v>15</v>
       </c>
       <c r="L15" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M15" s="62">
         <v>5.5E-2</v>
@@ -2159,19 +2159,19 @@
         <v>25</v>
       </c>
       <c r="E16" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G16" s="66" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="J16" s="36">
         <v>1</v>
@@ -2181,7 +2181,7 @@
         <v>5</v>
       </c>
       <c r="L16" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M16" s="61">
         <v>0.75</v>
@@ -2205,19 +2205,19 @@
         <v>26</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G17" s="67" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="J17" s="38">
         <v>2</v>
@@ -2227,13 +2227,13 @@
         <v>10</v>
       </c>
       <c r="L17" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M17" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="N17" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O17" s="38"/>
     </row>
@@ -2250,19 +2250,19 @@
         <v>27</v>
       </c>
       <c r="E18" s="36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G18" s="66" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J18" s="36">
         <v>2</v>
@@ -2272,7 +2272,7 @@
         <v>10</v>
       </c>
       <c r="L18" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M18" s="61">
         <v>9.7000000000000003E-2</v>
@@ -2296,19 +2296,19 @@
         <v>28</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G19" s="67" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="J19" s="38">
         <v>1</v>
@@ -2318,7 +2318,7 @@
         <v>5</v>
       </c>
       <c r="L19" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M19" s="62">
         <v>0.32</v>
@@ -2342,19 +2342,19 @@
         <v>29</v>
       </c>
       <c r="E20" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G20" s="66" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J20" s="36">
         <v>1</v>
@@ -2364,11 +2364,11 @@
         <v>5</v>
       </c>
       <c r="L20" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M20" s="61"/>
       <c r="N20" s="61" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O20" s="36"/>
     </row>
@@ -2385,19 +2385,19 @@
         <v>30</v>
       </c>
       <c r="E21" s="38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G21" s="67" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J21" s="38">
         <v>1</v>
@@ -2407,11 +2407,11 @@
         <v>5</v>
       </c>
       <c r="L21" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M21" s="62"/>
       <c r="N21" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O21" s="38"/>
     </row>
@@ -2428,19 +2428,19 @@
         <v>31</v>
       </c>
       <c r="E22" s="36" t="s">
-        <v>72</v>
+        <v>228</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="G22" s="66" t="s">
-        <v>132</v>
+        <v>105</v>
+      </c>
+      <c r="G22" s="36" t="s">
+        <v>229</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J22" s="36">
         <v>1</v>
@@ -2450,11 +2450,11 @@
         <v>5</v>
       </c>
       <c r="L22" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M22" s="61"/>
       <c r="N22" s="61" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O22" s="36"/>
     </row>
@@ -2471,19 +2471,19 @@
         <v>32</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G23" s="67" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J23" s="38">
         <v>2</v>
@@ -2493,7 +2493,7 @@
         <v>10</v>
       </c>
       <c r="L23" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M23" s="62">
         <v>0.38</v>
@@ -2511,25 +2511,25 @@
         <v>15</v>
       </c>
       <c r="C24" s="55" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D24" s="58" t="s">
         <v>33</v>
       </c>
       <c r="E24" s="58" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F24" s="59" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G24" s="58" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H24" s="58" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="I24" s="58" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J24" s="36">
         <v>1</v>
@@ -2539,13 +2539,13 @@
         <v>5</v>
       </c>
       <c r="L24" s="36" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="M24" s="63" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="N24" s="63" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O24" s="36"/>
     </row>
@@ -2562,19 +2562,19 @@
         <v>34</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G25" s="38" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J25" s="38">
         <v>1</v>
@@ -2584,7 +2584,7 @@
         <v>5</v>
       </c>
       <c r="L25" s="60" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="M25" s="62">
         <v>3.47</v>
@@ -2608,19 +2608,19 @@
         <v>35</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F26" s="38" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G26" s="66" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="J26" s="36">
         <v>1</v>
@@ -2630,11 +2630,11 @@
         <v>5</v>
       </c>
       <c r="L26" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M26" s="61"/>
       <c r="N26" s="61" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O26" s="36"/>
     </row>
@@ -2651,19 +2651,19 @@
         <v>36</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G27" s="67" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J27" s="38">
         <v>1</v>
@@ -2673,11 +2673,11 @@
         <v>5</v>
       </c>
       <c r="L27" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M27" s="62"/>
       <c r="N27" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O27" s="38"/>
     </row>
@@ -2694,19 +2694,19 @@
         <v>37</v>
       </c>
       <c r="E28" s="36" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G28" s="66" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="I28" s="38" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J28" s="36">
         <v>1</v>
@@ -2716,7 +2716,7 @@
         <v>5</v>
       </c>
       <c r="L28" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M28" s="61">
         <v>0.46</v>
@@ -2740,19 +2740,19 @@
         <v>38</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G29" s="67" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="J29" s="38">
         <v>1</v>
@@ -2762,11 +2762,11 @@
         <v>5</v>
       </c>
       <c r="L29" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M29" s="62"/>
       <c r="N29" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O29" s="38"/>
     </row>
@@ -2783,19 +2783,19 @@
         <v>39</v>
       </c>
       <c r="E30" s="36" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G30" s="66" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="J30" s="36">
         <v>1</v>
@@ -2805,7 +2805,7 @@
         <v>5</v>
       </c>
       <c r="L30" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M30" s="61">
         <v>0.2155</v>
@@ -2826,39 +2826,39 @@
         <v>14</v>
       </c>
       <c r="D31" s="38" t="s">
-        <v>40</v>
+        <v>231</v>
       </c>
       <c r="E31" s="38" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G31" s="67" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I31" s="38" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="J31" s="38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K31" s="39">
         <f t="shared" ref="K31" si="16">J31*5</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L31" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M31" s="62">
         <v>0.1</v>
       </c>
       <c r="N31" s="62">
         <f t="shared" ref="N31" si="17">M31*K31</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O31" s="38"/>
     </row>
@@ -2872,22 +2872,22 @@
         <v>14</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E32" s="36" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G32" s="66" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="J32" s="36">
         <v>1</v>
@@ -2897,7 +2897,7 @@
         <v>5</v>
       </c>
       <c r="L32" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M32" s="61">
         <v>0.9</v>
@@ -2918,22 +2918,22 @@
         <v>14</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G33" s="67" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="J33" s="38">
         <v>1</v>
@@ -2943,7 +2943,7 @@
         <v>5</v>
       </c>
       <c r="L33" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M33" s="62">
         <v>0.1</v>
@@ -2964,22 +2964,22 @@
         <v>14</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E34" s="36" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G34" s="66" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="J34" s="36">
         <v>1</v>
@@ -2989,11 +2989,11 @@
         <v>5</v>
       </c>
       <c r="L34" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M34" s="61"/>
       <c r="N34" s="61" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O34" s="36"/>
     </row>
@@ -3007,22 +3007,22 @@
         <v>14</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E35" s="38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G35" s="66" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I35" s="38" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="J35" s="38">
         <v>1</v>
@@ -3032,7 +3032,7 @@
         <v>5</v>
       </c>
       <c r="L35" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M35" s="62">
         <v>0.15</v>
@@ -3053,22 +3053,22 @@
         <v>14</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G36" s="66" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="H36" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="J36" s="36">
         <v>1</v>
@@ -3078,7 +3078,7 @@
         <v>5</v>
       </c>
       <c r="L36" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M36" s="61">
         <v>0.1</v>
@@ -3099,22 +3099,22 @@
         <v>14</v>
       </c>
       <c r="D37" s="38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F37" s="38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G37" s="67" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="J37" s="38">
         <v>1</v>
@@ -3124,7 +3124,7 @@
         <v>5</v>
       </c>
       <c r="L37" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M37" s="61">
         <v>0.1</v>
@@ -3145,22 +3145,22 @@
         <v>14</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E38" s="36" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G38" s="66" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H38" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="J38" s="36">
         <v>13</v>
@@ -3170,7 +3170,7 @@
         <v>65</v>
       </c>
       <c r="L38" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M38" s="61">
         <v>1.6199999999999999E-2</v>
@@ -3184,140 +3184,140 @@
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="56">
-        <f t="shared" si="0"/>
+        <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
       <c r="C39" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>47</v>
+        <v>227</v>
       </c>
       <c r="E39" s="38" t="s">
         <v>88</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G39" s="67" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I39" s="38" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J39" s="38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K39" s="39">
         <f t="shared" ref="K39" si="24">J39*5</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="L39" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M39" s="62">
-        <v>0.1</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="N39" s="62">
         <f t="shared" ref="N39" si="25">M39*K39</f>
-        <v>0.5</v>
+        <v>0.26999999999999996</v>
       </c>
       <c r="O39" s="38"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="54">
-        <f>ROW(B40) - ROW($B$9)</f>
+      <c r="B40" s="56">
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="55" t="s">
+      <c r="C40" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="D40" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="E40" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="F40" s="36" t="s">
-        <v>115</v>
-      </c>
-      <c r="G40" s="66" t="s">
-        <v>148</v>
-      </c>
-      <c r="H40" s="36" t="s">
-        <v>162</v>
-      </c>
-      <c r="I40" s="36" t="s">
-        <v>201</v>
-      </c>
-      <c r="J40" s="36">
-        <v>2</v>
-      </c>
-      <c r="K40" s="37">
-        <f>J40*5</f>
-        <v>10</v>
+      <c r="D40" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="E40" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="F40" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="G40" s="67" t="s">
+        <v>144</v>
+      </c>
+      <c r="H40" s="38" t="s">
+        <v>159</v>
+      </c>
+      <c r="I40" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="J40" s="38">
+        <v>1</v>
+      </c>
+      <c r="K40" s="39">
+        <f t="shared" ref="K40" si="26">J40*5</f>
+        <v>5</v>
       </c>
       <c r="L40" s="60" t="s">
-        <v>217</v>
-      </c>
-      <c r="M40" s="61">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="N40" s="61">
-        <f>M40*K40</f>
-        <v>0.15</v>
-      </c>
-      <c r="O40" s="36"/>
+        <v>213</v>
+      </c>
+      <c r="M40" s="62">
+        <v>0.1</v>
+      </c>
+      <c r="N40" s="62">
+        <f t="shared" ref="N40" si="27">M40*K40</f>
+        <v>0.5</v>
+      </c>
+      <c r="O40" s="38"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="56">
-        <f t="shared" si="0"/>
+      <c r="B41" s="54">
+        <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
-      <c r="C41" s="57" t="s">
+      <c r="C41" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="38" t="s">
-        <v>231</v>
-      </c>
-      <c r="E41" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="F41" s="38" t="s">
-        <v>115</v>
-      </c>
-      <c r="G41" s="67" t="s">
-        <v>149</v>
-      </c>
-      <c r="H41" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="I41" s="38" t="s">
-        <v>202</v>
-      </c>
-      <c r="J41" s="38">
-        <v>3</v>
-      </c>
-      <c r="K41" s="39">
-        <f t="shared" ref="K41" si="26">J41*5</f>
-        <v>15</v>
+      <c r="D41" s="36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E41" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="F41" s="36" t="s">
+        <v>113</v>
+      </c>
+      <c r="G41" s="66" t="s">
+        <v>145</v>
+      </c>
+      <c r="H41" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="I41" s="36" t="s">
+        <v>197</v>
+      </c>
+      <c r="J41" s="36">
+        <v>2</v>
+      </c>
+      <c r="K41" s="37">
+        <f>J41*5</f>
+        <v>10</v>
       </c>
       <c r="L41" s="60" t="s">
-        <v>217</v>
-      </c>
-      <c r="M41" s="62">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="N41" s="62">
-        <f t="shared" ref="N41" si="27">M41*K41</f>
-        <v>0.26999999999999996</v>
-      </c>
-      <c r="O41" s="38"/>
+        <v>213</v>
+      </c>
+      <c r="M41" s="61">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="N41" s="61">
+        <f>M41*K41</f>
+        <v>0.15</v>
+      </c>
+      <c r="O41" s="36"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
@@ -3329,22 +3329,22 @@
         <v>14</v>
       </c>
       <c r="D42" s="36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E42" s="36" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G42" s="66" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H42" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="J42" s="36">
         <v>4</v>
@@ -3354,7 +3354,7 @@
         <v>20</v>
       </c>
       <c r="L42" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M42" s="61">
         <v>2.5999999999999999E-2</v>
@@ -3375,22 +3375,22 @@
         <v>14</v>
       </c>
       <c r="D43" s="38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E43" s="38" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F43" s="38" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G43" s="67" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I43" s="38" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="J43" s="38">
         <v>1</v>
@@ -3400,7 +3400,7 @@
         <v>5</v>
       </c>
       <c r="L43" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M43" s="62">
         <v>0.1</v>
@@ -3421,22 +3421,22 @@
         <v>14</v>
       </c>
       <c r="D44" s="36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E44" s="36" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G44" s="66" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H44" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="J44" s="36">
         <v>4</v>
@@ -3446,7 +3446,7 @@
         <v>20</v>
       </c>
       <c r="L44" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M44" s="61">
         <v>1.7999999999999999E-2</v>
@@ -3467,22 +3467,22 @@
         <v>14</v>
       </c>
       <c r="D45" s="38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E45" s="38" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F45" s="38" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G45" s="67" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H45" s="38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I45" s="38" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="J45" s="38">
         <v>1</v>
@@ -3492,7 +3492,7 @@
         <v>5</v>
       </c>
       <c r="L45" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M45" s="62">
         <v>0.1</v>
@@ -3513,22 +3513,22 @@
         <v>14</v>
       </c>
       <c r="D46" s="36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E46" s="36" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F46" s="36" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G46" s="66" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H46" s="36" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I46" s="36" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="J46" s="36">
         <v>1</v>
@@ -3538,7 +3538,7 @@
         <v>5</v>
       </c>
       <c r="L46" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M46" s="61">
         <v>0.1</v>
@@ -3559,22 +3559,22 @@
         <v>15</v>
       </c>
       <c r="D47" s="38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E47" s="38" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="F47" s="38" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G47" s="38" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="H47" s="38" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="I47" s="38" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J47" s="38">
         <v>1</v>
@@ -3584,7 +3584,7 @@
         <v>5</v>
       </c>
       <c r="L47" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M47" s="62">
         <v>2.97</v>
@@ -3605,22 +3605,22 @@
         <v>15</v>
       </c>
       <c r="D48" s="36" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E48" s="36" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G48" s="66" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="H48" s="36" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J48" s="36">
         <v>1</v>
@@ -3630,11 +3630,11 @@
         <v>5</v>
       </c>
       <c r="L48" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M48" s="61"/>
       <c r="N48" s="61" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O48" s="36"/>
     </row>
@@ -3648,22 +3648,22 @@
         <v>15</v>
       </c>
       <c r="D49" s="38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E49" s="38" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F49" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G49" s="67" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H49" s="38" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="I49" s="38" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J49" s="38">
         <v>1</v>
@@ -3673,11 +3673,11 @@
         <v>5</v>
       </c>
       <c r="L49" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M49" s="62"/>
       <c r="N49" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O49" s="38"/>
     </row>
@@ -3691,22 +3691,22 @@
         <v>16</v>
       </c>
       <c r="D50" s="36" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E50" s="36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G50" s="66" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H50" s="36" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="I50" s="36" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J50" s="36">
         <v>1</v>
@@ -3716,7 +3716,7 @@
         <v>5</v>
       </c>
       <c r="L50" s="60" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="M50" s="61">
         <v>0.87</v>
@@ -3737,22 +3737,22 @@
         <v>17</v>
       </c>
       <c r="D51" s="38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E51" s="38" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F51" s="38" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G51" s="38" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H51" s="38" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="I51" s="36" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J51" s="38">
         <v>1</v>
@@ -3762,11 +3762,11 @@
         <v>5</v>
       </c>
       <c r="L51" s="60" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M51" s="62"/>
       <c r="N51" s="62" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="O51" s="38"/>
     </row>
@@ -3786,7 +3786,7 @@
       <c r="M52" s="35"/>
       <c r="N52" s="64">
         <f>SUM(N10:N51)</f>
-        <v>76.320499999999996</v>
+        <v>76.820499999999996</v>
       </c>
       <c r="O52" s="41"/>
     </row>
@@ -3806,7 +3806,7 @@
       <c r="M53" s="9"/>
       <c r="N53" s="65">
         <f>N52/5</f>
-        <v>15.264099999999999</v>
+        <v>15.364099999999999</v>
       </c>
       <c r="O53" s="42"/>
     </row>
@@ -3834,9 +3834,9 @@
     <hyperlink ref="L36" r:id="rId16"/>
     <hyperlink ref="L37" r:id="rId17"/>
     <hyperlink ref="L38" r:id="rId18"/>
-    <hyperlink ref="L39" r:id="rId19"/>
-    <hyperlink ref="L40" r:id="rId20"/>
-    <hyperlink ref="L41" r:id="rId21"/>
+    <hyperlink ref="L40" r:id="rId19"/>
+    <hyperlink ref="L41" r:id="rId20"/>
+    <hyperlink ref="L39" r:id="rId21"/>
     <hyperlink ref="L42" r:id="rId22"/>
     <hyperlink ref="L43" r:id="rId23"/>
     <hyperlink ref="L44" r:id="rId24"/>

</xml_diff>

<commit_message>
#18 Client BOM Updated.
</commit_message>
<xml_diff>
--- a/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
+++ b/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="234">
   <si>
     <t>Component list</t>
   </si>
@@ -189,9 +189,6 @@
     <t>U3</t>
   </si>
   <si>
-    <t>U4</t>
-  </si>
-  <si>
     <t>X1</t>
   </si>
   <si>
@@ -309,9 +306,6 @@
     <t>SPI LQFP-48(7x7) Ethernet ICs ROHS</t>
   </si>
   <si>
-    <t>TVS DIODE 5.5VWM 8.5VC SOT23-5</t>
-  </si>
-  <si>
     <t>SMD3225-4P Crystals ROHS</t>
   </si>
   <si>
@@ -369,9 +363,6 @@
     <t>48-LQFP (7x7)_</t>
   </si>
   <si>
-    <t>SOT-23-5</t>
-  </si>
-  <si>
     <t>NX3225GA-25MHZ-STD-CRG-2</t>
   </si>
   <si>
@@ -483,9 +474,6 @@
     <t>W5500</t>
   </si>
   <si>
-    <t>SP0504BAHTG</t>
-  </si>
-  <si>
     <t>Manufacturer</t>
   </si>
   <si>
@@ -724,6 +712,15 @@
   </si>
   <si>
     <t xml:space="preserve">Shengwei </t>
+  </si>
+  <si>
+    <t>D3, D4</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5.5VWM 8.5VC SOT23-3</t>
+  </si>
+  <si>
+    <t>SP0502BAHTG</t>
   </si>
 </sst>
 </file>
@@ -1313,6 +1310,12 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1321,12 +1324,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1698,13 +1695,13 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
     </row>
     <row r="2" spans="1:15" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1715,7 +1712,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="50" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1736,7 +1733,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="51" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1746,7 +1743,7 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
-      <c r="O3" s="69"/>
+      <c r="O3" s="71"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1757,7 +1754,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="52" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1767,7 +1764,7 @@
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
-      <c r="O4" s="70"/>
+      <c r="O4" s="72"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1788,7 +1785,7 @@
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
-      <c r="O5" s="70"/>
+      <c r="O5" s="72"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1805,7 +1802,7 @@
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
-      <c r="O6" s="70"/>
+      <c r="O6" s="72"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1822,7 +1819,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
-      <c r="O7" s="70"/>
+      <c r="O7" s="72"/>
     </row>
     <row r="8" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1839,7 +1836,7 @@
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
-      <c r="O8" s="70"/>
+      <c r="O8" s="72"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1853,37 +1850,37 @@
         <v>18</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I9" s="30" t="s">
+        <v>203</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>204</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>206</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>207</v>
       </c>
-      <c r="J9" s="29" t="s">
-        <v>214</v>
-      </c>
-      <c r="K9" s="29" t="s">
+      <c r="N9" s="29" t="s">
         <v>208</v>
       </c>
-      <c r="L9" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>211</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>212</v>
-      </c>
       <c r="O9" s="29" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1899,19 +1896,19 @@
         <v>19</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="J10" s="36">
         <v>10</v>
@@ -1921,7 +1918,7 @@
         <v>50</v>
       </c>
       <c r="L10" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M10" s="61">
         <v>1.26E-2</v>
@@ -1945,19 +1942,19 @@
         <v>20</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="J11" s="38">
         <v>1</v>
@@ -1967,13 +1964,13 @@
         <v>5</v>
       </c>
       <c r="L11" s="60" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="M11" s="62" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="N11" s="62" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="O11" s="38"/>
     </row>
@@ -1990,19 +1987,19 @@
         <v>21</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G12" s="66" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J12" s="36">
         <v>3</v>
@@ -2012,7 +2009,7 @@
         <v>15</v>
       </c>
       <c r="L12" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M12" s="61">
         <v>7.0999999999999994E-2</v>
@@ -2036,19 +2033,19 @@
         <v>22</v>
       </c>
       <c r="E13" s="38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G13" s="67" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="J13" s="38">
         <v>1</v>
@@ -2058,7 +2055,7 @@
         <v>5</v>
       </c>
       <c r="L13" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M13" s="62">
         <v>2.33</v>
@@ -2082,19 +2079,19 @@
         <v>23</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G14" s="66" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="J14" s="36">
         <v>1</v>
@@ -2104,7 +2101,7 @@
         <v>5</v>
       </c>
       <c r="L14" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M14" s="61">
         <v>0.1</v>
@@ -2128,19 +2125,19 @@
         <v>24</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G15" s="66" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="J15" s="38">
         <v>3</v>
@@ -2150,7 +2147,7 @@
         <v>15</v>
       </c>
       <c r="L15" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M15" s="62">
         <v>5.5E-2</v>
@@ -2174,19 +2171,19 @@
         <v>25</v>
       </c>
       <c r="E16" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G16" s="66" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="J16" s="36">
         <v>1</v>
@@ -2196,7 +2193,7 @@
         <v>5</v>
       </c>
       <c r="L16" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M16" s="61">
         <v>0.75</v>
@@ -2220,19 +2217,19 @@
         <v>26</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G17" s="67" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J17" s="38">
         <v>2</v>
@@ -2242,13 +2239,13 @@
         <v>10</v>
       </c>
       <c r="L17" s="60" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="M17" s="62" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="N17" s="62" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="O17" s="38"/>
     </row>
@@ -2265,19 +2262,19 @@
         <v>27</v>
       </c>
       <c r="E18" s="36" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G18" s="66" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="J18" s="36">
         <v>2</v>
@@ -2287,7 +2284,7 @@
         <v>10</v>
       </c>
       <c r="L18" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M18" s="61">
         <v>9.7000000000000003E-2</v>
@@ -2311,19 +2308,19 @@
         <v>28</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G19" s="67" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J19" s="38">
         <v>1</v>
@@ -2333,13 +2330,13 @@
         <v>5</v>
       </c>
       <c r="L19" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M19" s="62">
         <v>0.32</v>
       </c>
       <c r="N19" s="62">
-        <f t="shared" ref="N19" si="8">M19*K19</f>
+        <f t="shared" ref="N19:N22" si="8">M19*K19</f>
         <v>1.6</v>
       </c>
       <c r="O19" s="38"/>
@@ -2357,19 +2354,19 @@
         <v>29</v>
       </c>
       <c r="E20" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G20" s="66" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="J20" s="36">
         <v>1</v>
@@ -2379,12 +2376,10 @@
         <v>5</v>
       </c>
       <c r="L20" s="60" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="M20" s="61"/>
-      <c r="N20" s="61" t="s">
-        <v>206</v>
-      </c>
+      <c r="N20" s="62"/>
       <c r="O20" s="36"/>
     </row>
     <row r="21" spans="1:15" ht="30" x14ac:dyDescent="0.25">
@@ -2400,939 +2395,937 @@
         <v>30</v>
       </c>
       <c r="E21" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G21" s="67" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="J21" s="38">
         <v>1</v>
       </c>
       <c r="K21" s="39">
-        <f t="shared" ref="K21" si="9">J21*5</f>
+        <f t="shared" ref="K21:K22" si="9">J21*5</f>
         <v>5</v>
       </c>
       <c r="L21" s="60" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="M21" s="62"/>
-      <c r="N21" s="62" t="s">
-        <v>206</v>
-      </c>
+      <c r="N21" s="62"/>
       <c r="O21" s="38"/>
     </row>
-    <row r="22" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="54">
-        <f>ROW(B22) - ROW($B$9)</f>
+      <c r="B22" s="56">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C22" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="E22" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="F22" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="G22" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="H22" s="36" t="s">
+        <v>169</v>
+      </c>
+      <c r="I22" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="J22" s="36">
+        <v>2</v>
+      </c>
+      <c r="K22" s="37">
+        <f t="shared" si="9"/>
+        <v>10</v>
+      </c>
+      <c r="L22" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M22" s="61">
+        <v>0.57799999999999996</v>
+      </c>
+      <c r="N22" s="62">
+        <f t="shared" si="8"/>
+        <v>5.7799999999999994</v>
+      </c>
+      <c r="O22" s="36"/>
+    </row>
+    <row r="23" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="54">
+        <f>ROW(B23) - ROW($B$9)</f>
+        <v>14</v>
+      </c>
+      <c r="C23" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="36" t="s">
+      <c r="D23" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="F22" s="36" t="s">
-        <v>105</v>
-      </c>
-      <c r="G22" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="H22" s="36" t="s">
-        <v>230</v>
-      </c>
-      <c r="I22" s="36" t="s">
-        <v>206</v>
-      </c>
-      <c r="J22" s="36">
+      <c r="E23" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="F23" s="36" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="H23" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="I23" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="J23" s="36">
         <v>1</v>
       </c>
-      <c r="K22" s="37">
-        <f>J22*5</f>
+      <c r="K23" s="37">
+        <f>J23*5</f>
         <v>5</v>
       </c>
-      <c r="L22" s="60" t="s">
-        <v>218</v>
-      </c>
-      <c r="M22" s="61"/>
-      <c r="N22" s="61" t="s">
-        <v>206</v>
-      </c>
-      <c r="O22" s="36"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="56">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="C23" s="57" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>71</v>
-      </c>
-      <c r="F23" s="38" t="s">
-        <v>106</v>
-      </c>
-      <c r="G23" s="67" t="s">
-        <v>130</v>
-      </c>
-      <c r="H23" s="38" t="s">
-        <v>164</v>
-      </c>
-      <c r="I23" s="38" t="s">
-        <v>206</v>
-      </c>
-      <c r="J23" s="38">
-        <v>2</v>
-      </c>
-      <c r="K23" s="39">
-        <f t="shared" ref="K23" si="10">J23*5</f>
-        <v>10</v>
-      </c>
       <c r="L23" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M23" s="62">
-        <v>0.38</v>
-      </c>
-      <c r="N23" s="62">
-        <f t="shared" ref="N23" si="11">M23*K23</f>
-        <v>3.8</v>
-      </c>
-      <c r="O23" s="38"/>
+        <v>214</v>
+      </c>
+      <c r="M23" s="61"/>
+      <c r="N23" s="61" t="s">
+        <v>202</v>
+      </c>
+      <c r="O23" s="36"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="54">
-        <f>ROW(B24) - ROW($B$9)</f>
+      <c r="B24" s="56">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="55" t="s">
-        <v>205</v>
-      </c>
-      <c r="D24" s="58" t="s">
-        <v>33</v>
-      </c>
-      <c r="E24" s="58" t="s">
-        <v>72</v>
-      </c>
-      <c r="F24" s="59" t="s">
-        <v>204</v>
-      </c>
-      <c r="G24" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="H24" s="58" t="s">
-        <v>206</v>
-      </c>
-      <c r="I24" s="58" t="s">
-        <v>206</v>
-      </c>
-      <c r="J24" s="36">
-        <v>1</v>
-      </c>
-      <c r="K24" s="37">
-        <f>J24*5</f>
-        <v>5</v>
-      </c>
-      <c r="L24" s="36" t="s">
-        <v>206</v>
-      </c>
-      <c r="M24" s="63" t="s">
-        <v>206</v>
-      </c>
-      <c r="N24" s="63" t="s">
-        <v>206</v>
-      </c>
-      <c r="O24" s="36"/>
+      <c r="C24" s="57" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24" s="38" t="s">
+        <v>70</v>
+      </c>
+      <c r="F24" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="G24" s="67" t="s">
+        <v>127</v>
+      </c>
+      <c r="H24" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="I24" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="J24" s="38">
+        <v>2</v>
+      </c>
+      <c r="K24" s="39">
+        <f t="shared" ref="K24" si="10">J24*5</f>
+        <v>10</v>
+      </c>
+      <c r="L24" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M24" s="62">
+        <v>0.38</v>
+      </c>
+      <c r="N24" s="62">
+        <f t="shared" ref="N24" si="11">M24*K24</f>
+        <v>3.8</v>
+      </c>
+      <c r="O24" s="38"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="56">
+      <c r="B25" s="54">
+        <f>ROW(B25) - ROW($B$9)</f>
+        <v>16</v>
+      </c>
+      <c r="C25" s="55" t="s">
+        <v>201</v>
+      </c>
+      <c r="D25" s="58" t="s">
+        <v>33</v>
+      </c>
+      <c r="E25" s="58" t="s">
+        <v>71</v>
+      </c>
+      <c r="F25" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="G25" s="58" t="s">
+        <v>105</v>
+      </c>
+      <c r="H25" s="58" t="s">
+        <v>202</v>
+      </c>
+      <c r="I25" s="58" t="s">
+        <v>202</v>
+      </c>
+      <c r="J25" s="36">
+        <v>1</v>
+      </c>
+      <c r="K25" s="37">
+        <f>J25*5</f>
+        <v>5</v>
+      </c>
+      <c r="L25" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="M25" s="63" t="s">
+        <v>202</v>
+      </c>
+      <c r="N25" s="63" t="s">
+        <v>202</v>
+      </c>
+      <c r="O25" s="36"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="56">
         <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="C25" s="57" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D26" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="E25" s="38" t="s">
-        <v>219</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>204</v>
-      </c>
-      <c r="G25" s="38" t="s">
-        <v>220</v>
-      </c>
-      <c r="H25" s="38" t="s">
-        <v>221</v>
-      </c>
-      <c r="I25" s="38" t="s">
-        <v>206</v>
-      </c>
-      <c r="J25" s="38">
+      <c r="E26" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>200</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="H26" s="38" t="s">
+        <v>217</v>
+      </c>
+      <c r="I26" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="J26" s="38">
         <v>1</v>
       </c>
-      <c r="K25" s="39">
-        <f t="shared" ref="K25" si="12">J25*5</f>
-        <v>5</v>
-      </c>
-      <c r="L25" s="60" t="s">
-        <v>222</v>
-      </c>
-      <c r="M25" s="62">
-        <v>3.47</v>
-      </c>
-      <c r="N25" s="62">
-        <f t="shared" ref="N25" si="13">M25*K25</f>
-        <v>17.350000000000001</v>
-      </c>
-      <c r="O25" s="38"/>
-    </row>
-    <row r="26" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="54">
-        <f>ROW(B26) - ROW($B$9)</f>
-        <v>17</v>
-      </c>
-      <c r="C26" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="36" t="s">
-        <v>73</v>
-      </c>
-      <c r="F26" s="38" t="s">
-        <v>204</v>
-      </c>
-      <c r="G26" s="66" t="s">
-        <v>131</v>
-      </c>
-      <c r="H26" s="36" t="s">
-        <v>165</v>
-      </c>
-      <c r="I26" s="36" t="s">
-        <v>185</v>
-      </c>
-      <c r="J26" s="36">
-        <v>1</v>
-      </c>
-      <c r="K26" s="37">
-        <f>J26*5</f>
+      <c r="K26" s="39">
+        <f t="shared" ref="K26" si="12">J26*5</f>
         <v>5</v>
       </c>
       <c r="L26" s="60" t="s">
         <v>218</v>
       </c>
-      <c r="M26" s="61"/>
-      <c r="N26" s="61" t="s">
-        <v>206</v>
-      </c>
-      <c r="O26" s="36"/>
-    </row>
-    <row r="27" spans="1:15" ht="48" x14ac:dyDescent="0.25">
+      <c r="M26" s="62">
+        <v>3.47</v>
+      </c>
+      <c r="N26" s="62">
+        <f t="shared" ref="N26" si="13">M26*K26</f>
+        <v>17.350000000000001</v>
+      </c>
+      <c r="O26" s="38"/>
+    </row>
+    <row r="27" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="56">
+      <c r="B27" s="54">
+        <f>ROW(B27) - ROW($B$9)</f>
+        <v>18</v>
+      </c>
+      <c r="C27" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="36" t="s">
+        <v>35</v>
+      </c>
+      <c r="E27" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="F27" s="38" t="s">
+        <v>200</v>
+      </c>
+      <c r="G27" s="66" t="s">
+        <v>128</v>
+      </c>
+      <c r="H27" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="I27" s="36" t="s">
+        <v>181</v>
+      </c>
+      <c r="J27" s="36">
+        <v>1</v>
+      </c>
+      <c r="K27" s="37">
+        <f>J27*5</f>
+        <v>5</v>
+      </c>
+      <c r="L27" s="60" t="s">
+        <v>214</v>
+      </c>
+      <c r="M27" s="61"/>
+      <c r="N27" s="61" t="s">
+        <v>202</v>
+      </c>
+      <c r="O27" s="36"/>
+    </row>
+    <row r="28" spans="1:15" ht="48" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="56">
         <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="C27" s="57" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="E27" s="38" t="s">
-        <v>74</v>
-      </c>
-      <c r="F27" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="G27" s="67" t="s">
-        <v>132</v>
-      </c>
-      <c r="H27" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="I27" s="36" t="s">
-        <v>206</v>
-      </c>
-      <c r="J27" s="38">
-        <v>1</v>
-      </c>
-      <c r="K27" s="39">
-        <f t="shared" ref="K27" si="14">J27*5</f>
-        <v>5</v>
-      </c>
-      <c r="L27" s="60" t="s">
-        <v>218</v>
-      </c>
-      <c r="M27" s="62"/>
-      <c r="N27" s="62" t="s">
-        <v>206</v>
-      </c>
-      <c r="O27" s="38"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
-      <c r="B28" s="54">
-        <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
       <c r="C28" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="D28" s="36" t="s">
+      <c r="D28" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="F28" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="G28" s="67" t="s">
+        <v>129</v>
+      </c>
+      <c r="H28" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="I28" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="J28" s="38">
+        <v>1</v>
+      </c>
+      <c r="K28" s="39">
+        <f t="shared" ref="K28" si="14">J28*5</f>
+        <v>5</v>
+      </c>
+      <c r="L28" s="60" t="s">
+        <v>214</v>
+      </c>
+      <c r="M28" s="62"/>
+      <c r="N28" s="62" t="s">
+        <v>202</v>
+      </c>
+      <c r="O28" s="38"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="54">
+        <f>ROW(B29) - ROW($B$9)</f>
+        <v>20</v>
+      </c>
+      <c r="C29" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="36" t="s">
+      <c r="E29" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="F29" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="G29" s="66" t="s">
+        <v>130</v>
+      </c>
+      <c r="H29" s="36" t="s">
+        <v>163</v>
+      </c>
+      <c r="I29" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="J29" s="36">
+        <v>1</v>
+      </c>
+      <c r="K29" s="37">
+        <f>J29*5</f>
+        <v>5</v>
+      </c>
+      <c r="L29" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M29" s="61">
+        <v>0.46</v>
+      </c>
+      <c r="N29" s="61">
+        <f>M29*K29</f>
+        <v>2.3000000000000003</v>
+      </c>
+      <c r="O29" s="36"/>
+    </row>
+    <row r="30" spans="1:15" ht="36" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="56">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="C30" s="57" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="38" t="s">
+        <v>38</v>
+      </c>
+      <c r="E30" s="38" t="s">
         <v>75</v>
       </c>
-      <c r="F28" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="G28" s="66" t="s">
-        <v>133</v>
-      </c>
-      <c r="H28" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="I28" s="38" t="s">
-        <v>206</v>
-      </c>
-      <c r="J28" s="36">
+      <c r="F30" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="G30" s="67" t="s">
+        <v>131</v>
+      </c>
+      <c r="H30" s="38" t="s">
+        <v>164</v>
+      </c>
+      <c r="I30" s="38" t="s">
+        <v>182</v>
+      </c>
+      <c r="J30" s="38">
         <v>1</v>
       </c>
-      <c r="K28" s="37">
-        <f>J28*5</f>
+      <c r="K30" s="39">
+        <f t="shared" ref="K30" si="15">J30*5</f>
         <v>5</v>
       </c>
-      <c r="L28" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M28" s="61">
-        <v>0.46</v>
-      </c>
-      <c r="N28" s="61">
-        <f>M28*K28</f>
-        <v>2.3000000000000003</v>
-      </c>
-      <c r="O28" s="36"/>
-    </row>
-    <row r="29" spans="1:15" ht="36" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="B29" s="56">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="C29" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="E29" s="38" t="s">
-        <v>76</v>
-      </c>
-      <c r="F29" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="G29" s="67" t="s">
-        <v>134</v>
-      </c>
-      <c r="H29" s="38" t="s">
-        <v>168</v>
-      </c>
-      <c r="I29" s="38" t="s">
-        <v>186</v>
-      </c>
-      <c r="J29" s="38">
-        <v>1</v>
-      </c>
-      <c r="K29" s="39">
-        <f t="shared" ref="K29" si="15">J29*5</f>
-        <v>5</v>
-      </c>
-      <c r="L29" s="60" t="s">
-        <v>218</v>
-      </c>
-      <c r="M29" s="62"/>
-      <c r="N29" s="62" t="s">
-        <v>206</v>
-      </c>
-      <c r="O29" s="38"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="B30" s="54">
-        <f>ROW(B30) - ROW($B$9)</f>
-        <v>21</v>
-      </c>
-      <c r="C30" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="D30" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E30" s="36" t="s">
-        <v>77</v>
-      </c>
-      <c r="F30" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="G30" s="66" t="s">
-        <v>135</v>
-      </c>
-      <c r="H30" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="I30" s="36" t="s">
-        <v>187</v>
-      </c>
-      <c r="J30" s="36">
-        <v>1</v>
-      </c>
-      <c r="K30" s="37">
-        <f>J30*5</f>
-        <v>5</v>
-      </c>
       <c r="L30" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M30" s="61">
-        <v>0.2155</v>
-      </c>
-      <c r="N30" s="61">
-        <f>M30*K30</f>
-        <v>1.0774999999999999</v>
-      </c>
-      <c r="O30" s="36"/>
+        <v>214</v>
+      </c>
+      <c r="M30" s="62"/>
+      <c r="N30" s="62" t="s">
+        <v>202</v>
+      </c>
+      <c r="O30" s="38"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="56">
-        <f t="shared" si="0"/>
+      <c r="B31" s="54">
+        <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="57" t="s">
+      <c r="C31" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="38" t="s">
-        <v>231</v>
-      </c>
-      <c r="E31" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="F31" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="G31" s="67" t="s">
-        <v>136</v>
-      </c>
-      <c r="H31" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="I31" s="38" t="s">
-        <v>188</v>
-      </c>
-      <c r="J31" s="38">
-        <v>2</v>
-      </c>
-      <c r="K31" s="39">
-        <f t="shared" ref="K31" si="16">J31*5</f>
-        <v>10</v>
+      <c r="D31" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="F31" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="G31" s="66" t="s">
+        <v>132</v>
+      </c>
+      <c r="H31" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="I31" s="36" t="s">
+        <v>183</v>
+      </c>
+      <c r="J31" s="36">
+        <v>1</v>
+      </c>
+      <c r="K31" s="37">
+        <f>J31*5</f>
+        <v>5</v>
       </c>
       <c r="L31" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M31" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N31" s="62">
-        <f t="shared" ref="N31" si="17">M31*K31</f>
-        <v>1</v>
-      </c>
-      <c r="O31" s="38"/>
+        <v>209</v>
+      </c>
+      <c r="M31" s="61">
+        <v>0.2155</v>
+      </c>
+      <c r="N31" s="61">
+        <f>M31*K31</f>
+        <v>1.0774999999999999</v>
+      </c>
+      <c r="O31" s="36"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="54">
-        <f>ROW(B32) - ROW($B$9)</f>
+      <c r="B32" s="56">
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="55" t="s">
+      <c r="C32" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="D32" s="36" t="s">
-        <v>40</v>
-      </c>
-      <c r="E32" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="F32" s="36" t="s">
-        <v>112</v>
-      </c>
-      <c r="G32" s="66" t="s">
-        <v>137</v>
-      </c>
-      <c r="H32" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="I32" s="36" t="s">
-        <v>189</v>
-      </c>
-      <c r="J32" s="36">
+      <c r="D32" s="38" t="s">
+        <v>227</v>
+      </c>
+      <c r="E32" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="F32" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="G32" s="67" t="s">
+        <v>133</v>
+      </c>
+      <c r="H32" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="I32" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="J32" s="38">
+        <v>2</v>
+      </c>
+      <c r="K32" s="39">
+        <f t="shared" ref="K32" si="16">J32*5</f>
+        <v>10</v>
+      </c>
+      <c r="L32" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M32" s="62">
+        <v>0.1</v>
+      </c>
+      <c r="N32" s="62">
+        <f t="shared" ref="N32" si="17">M32*K32</f>
         <v>1</v>
       </c>
-      <c r="K32" s="37">
-        <f>J32*5</f>
-        <v>5</v>
-      </c>
-      <c r="L32" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M32" s="61">
-        <v>0.9</v>
-      </c>
-      <c r="N32" s="61">
-        <f>M32*K32</f>
-        <v>4.5</v>
-      </c>
-      <c r="O32" s="36"/>
+      <c r="O32" s="38"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="56">
+      <c r="B33" s="54">
+        <f>ROW(B33) - ROW($B$9)</f>
+        <v>24</v>
+      </c>
+      <c r="C33" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="E33" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="F33" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="G33" s="66" t="s">
+        <v>134</v>
+      </c>
+      <c r="H33" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="I33" s="36" t="s">
+        <v>185</v>
+      </c>
+      <c r="J33" s="36">
+        <v>1</v>
+      </c>
+      <c r="K33" s="37">
+        <f>J33*5</f>
+        <v>5</v>
+      </c>
+      <c r="L33" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M33" s="61">
+        <v>0.9</v>
+      </c>
+      <c r="N33" s="61">
+        <f>M33*K33</f>
+        <v>4.5</v>
+      </c>
+      <c r="O33" s="36"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="56">
         <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="C33" s="57" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="D33" s="38" t="s">
+      <c r="D34" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="E33" s="38" t="s">
-        <v>80</v>
-      </c>
-      <c r="F33" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="G33" s="67" t="s">
-        <v>138</v>
-      </c>
-      <c r="H33" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="I33" s="38" t="s">
-        <v>190</v>
-      </c>
-      <c r="J33" s="38">
+      <c r="E34" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="F34" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="G34" s="67" t="s">
+        <v>135</v>
+      </c>
+      <c r="H34" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="I34" s="38" t="s">
+        <v>186</v>
+      </c>
+      <c r="J34" s="38">
         <v>1</v>
       </c>
-      <c r="K33" s="39">
-        <f t="shared" ref="K33" si="18">J33*5</f>
+      <c r="K34" s="39">
+        <f t="shared" ref="K34" si="18">J34*5</f>
         <v>5</v>
       </c>
-      <c r="L33" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M33" s="62">
+      <c r="L34" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M34" s="62">
         <v>0.1</v>
       </c>
-      <c r="N33" s="62">
-        <f t="shared" ref="N33" si="19">M33*K33</f>
+      <c r="N34" s="62">
+        <f t="shared" ref="N34" si="19">M34*K34</f>
         <v>0.5</v>
       </c>
-      <c r="O33" s="38"/>
-    </row>
-    <row r="34" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
-      <c r="B34" s="54">
-        <f>ROW(B34) - ROW($B$9)</f>
-        <v>25</v>
-      </c>
-      <c r="C34" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="36" t="s">
-        <v>42</v>
-      </c>
-      <c r="E34" s="36" t="s">
-        <v>81</v>
-      </c>
-      <c r="F34" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="G34" s="66" t="s">
-        <v>139</v>
-      </c>
-      <c r="H34" s="36" t="s">
-        <v>168</v>
-      </c>
-      <c r="I34" s="36" t="s">
-        <v>191</v>
-      </c>
-      <c r="J34" s="36">
-        <v>1</v>
-      </c>
-      <c r="K34" s="37">
-        <f>J34*5</f>
-        <v>5</v>
-      </c>
-      <c r="L34" s="60" t="s">
-        <v>218</v>
-      </c>
-      <c r="M34" s="61"/>
-      <c r="N34" s="61" t="s">
-        <v>206</v>
-      </c>
-      <c r="O34" s="36"/>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O34" s="38"/>
+    </row>
+    <row r="35" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="56">
-        <f t="shared" si="0"/>
+      <c r="B35" s="54">
+        <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
       <c r="C35" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D35" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="E35" s="38" t="s">
-        <v>82</v>
-      </c>
-      <c r="F35" s="38" t="s">
-        <v>113</v>
+      <c r="D35" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="F35" s="36" t="s">
+        <v>108</v>
       </c>
       <c r="G35" s="66" t="s">
-        <v>140</v>
-      </c>
-      <c r="H35" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="I35" s="38" t="s">
-        <v>192</v>
-      </c>
-      <c r="J35" s="38">
+        <v>136</v>
+      </c>
+      <c r="H35" s="36" t="s">
+        <v>164</v>
+      </c>
+      <c r="I35" s="36" t="s">
+        <v>187</v>
+      </c>
+      <c r="J35" s="36">
         <v>1</v>
       </c>
-      <c r="K35" s="39">
-        <f t="shared" ref="K35" si="20">J35*5</f>
+      <c r="K35" s="37">
+        <f>J35*5</f>
         <v>5</v>
       </c>
       <c r="L35" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M35" s="62">
-        <v>0.15</v>
-      </c>
-      <c r="N35" s="62">
-        <f t="shared" ref="N35" si="21">M35*K35</f>
-        <v>0.75</v>
-      </c>
-      <c r="O35" s="38"/>
+        <v>214</v>
+      </c>
+      <c r="M35" s="61"/>
+      <c r="N35" s="61" t="s">
+        <v>202</v>
+      </c>
+      <c r="O35" s="36"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="54">
-        <f>ROW(B36) - ROW($B$9)</f>
+      <c r="B36" s="56">
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C36" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D36" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="E36" s="36" t="s">
-        <v>83</v>
-      </c>
-      <c r="F36" s="36" t="s">
-        <v>110</v>
+      <c r="D36" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="E36" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="F36" s="38" t="s">
+        <v>111</v>
       </c>
       <c r="G36" s="66" t="s">
-        <v>141</v>
-      </c>
-      <c r="H36" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="I36" s="36" t="s">
-        <v>193</v>
-      </c>
-      <c r="J36" s="36">
+        <v>137</v>
+      </c>
+      <c r="H36" s="38" t="s">
+        <v>165</v>
+      </c>
+      <c r="I36" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="J36" s="38">
         <v>1</v>
       </c>
-      <c r="K36" s="37">
-        <f>J36*5</f>
+      <c r="K36" s="39">
+        <f t="shared" ref="K36" si="20">J36*5</f>
         <v>5</v>
       </c>
       <c r="L36" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M36" s="61">
-        <v>0.1</v>
-      </c>
-      <c r="N36" s="61">
-        <f>M36*K36</f>
-        <v>0.5</v>
-      </c>
-      <c r="O36" s="36"/>
+        <v>209</v>
+      </c>
+      <c r="M36" s="62">
+        <v>0.15</v>
+      </c>
+      <c r="N36" s="62">
+        <f t="shared" ref="N36" si="21">M36*K36</f>
+        <v>0.75</v>
+      </c>
+      <c r="O36" s="38"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="56">
-        <f t="shared" si="0"/>
+      <c r="B37" s="54">
+        <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
-      <c r="C37" s="57" t="s">
+      <c r="C37" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D37" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="E37" s="38" t="s">
-        <v>84</v>
-      </c>
-      <c r="F37" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="G37" s="67" t="s">
-        <v>142</v>
-      </c>
-      <c r="H37" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="I37" s="38" t="s">
-        <v>194</v>
-      </c>
-      <c r="J37" s="38">
+      <c r="D37" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="E37" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="F37" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="G37" s="66" t="s">
+        <v>138</v>
+      </c>
+      <c r="H37" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="I37" s="36" t="s">
+        <v>189</v>
+      </c>
+      <c r="J37" s="36">
         <v>1</v>
       </c>
-      <c r="K37" s="39">
-        <f t="shared" ref="K37" si="22">J37*5</f>
+      <c r="K37" s="37">
+        <f>J37*5</f>
         <v>5</v>
       </c>
       <c r="L37" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M37" s="61">
         <v>0.1</v>
       </c>
-      <c r="N37" s="62">
-        <f t="shared" ref="N37" si="23">M37*K37</f>
+      <c r="N37" s="61">
+        <f>M37*K37</f>
         <v>0.5</v>
       </c>
-      <c r="O37" s="38"/>
-    </row>
-    <row r="38" spans="1:15" ht="24" x14ac:dyDescent="0.25">
+      <c r="O37" s="36"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="54">
-        <f>ROW(B38) - ROW($B$9)</f>
+      <c r="B38" s="56">
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="55" t="s">
+      <c r="C38" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="D38" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="E38" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="F38" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="G38" s="66" t="s">
-        <v>143</v>
-      </c>
-      <c r="H38" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="I38" s="36" t="s">
-        <v>195</v>
-      </c>
-      <c r="J38" s="36">
-        <v>13</v>
-      </c>
-      <c r="K38" s="37">
-        <f>J38*5</f>
-        <v>65</v>
+      <c r="D38" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="E38" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="F38" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="G38" s="67" t="s">
+        <v>139</v>
+      </c>
+      <c r="H38" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="I38" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="J38" s="38">
+        <v>1</v>
+      </c>
+      <c r="K38" s="39">
+        <f t="shared" ref="K38" si="22">J38*5</f>
+        <v>5</v>
       </c>
       <c r="L38" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M38" s="61">
-        <v>1.6199999999999999E-2</v>
-      </c>
-      <c r="N38" s="61">
-        <f>M38*K38</f>
-        <v>1.0529999999999999</v>
-      </c>
-      <c r="O38" s="36"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+      <c r="N38" s="62">
+        <f t="shared" ref="N38" si="23">M38*K38</f>
+        <v>0.5</v>
+      </c>
+      <c r="O38" s="38"/>
+    </row>
+    <row r="39" spans="1:15" ht="24" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="56">
+      <c r="B39" s="54">
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="57" t="s">
+      <c r="C39" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="38" t="s">
-        <v>227</v>
-      </c>
-      <c r="E39" s="38" t="s">
-        <v>88</v>
-      </c>
-      <c r="F39" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="G39" s="67" t="s">
-        <v>146</v>
-      </c>
-      <c r="H39" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="I39" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="J39" s="38">
-        <v>3</v>
-      </c>
-      <c r="K39" s="39">
-        <f t="shared" ref="K39" si="24">J39*5</f>
-        <v>15</v>
+      <c r="D39" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="E39" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="F39" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="G39" s="66" t="s">
+        <v>140</v>
+      </c>
+      <c r="H39" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="I39" s="36" t="s">
+        <v>191</v>
+      </c>
+      <c r="J39" s="36">
+        <v>13</v>
+      </c>
+      <c r="K39" s="37">
+        <f>J39*5</f>
+        <v>65</v>
       </c>
       <c r="L39" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M39" s="62">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="N39" s="62">
-        <f t="shared" ref="N39" si="25">M39*K39</f>
-        <v>0.26999999999999996</v>
-      </c>
-      <c r="O39" s="38"/>
+        <v>209</v>
+      </c>
+      <c r="M39" s="61">
+        <v>1.6199999999999999E-2</v>
+      </c>
+      <c r="N39" s="61">
+        <f>M39*K39</f>
+        <v>1.0529999999999999</v>
+      </c>
+      <c r="O39" s="36"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="56">
-        <f t="shared" si="0"/>
+        <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
       <c r="C40" s="57" t="s">
         <v>14</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>46</v>
+        <v>223</v>
       </c>
       <c r="E40" s="38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F40" s="38" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G40" s="67" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H40" s="38" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I40" s="38" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="J40" s="38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K40" s="39">
-        <f t="shared" ref="K40" si="26">J40*5</f>
-        <v>5</v>
+        <f t="shared" ref="K40" si="24">J40*5</f>
+        <v>15</v>
       </c>
       <c r="L40" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M40" s="62">
-        <v>0.1</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="N40" s="62">
-        <f t="shared" ref="N40" si="27">M40*K40</f>
-        <v>0.5</v>
+        <f t="shared" ref="N40" si="25">M40*K40</f>
+        <v>0.26999999999999996</v>
       </c>
       <c r="O40" s="38"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="54">
-        <f>ROW(B41) - ROW($B$9)</f>
+      <c r="B41" s="56">
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="55" t="s">
+      <c r="C41" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="36" t="s">
-        <v>47</v>
-      </c>
-      <c r="E41" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="F41" s="36" t="s">
-        <v>113</v>
-      </c>
-      <c r="G41" s="66" t="s">
-        <v>145</v>
-      </c>
-      <c r="H41" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="I41" s="36" t="s">
-        <v>197</v>
-      </c>
-      <c r="J41" s="36">
-        <v>2</v>
-      </c>
-      <c r="K41" s="37">
-        <f>J41*5</f>
-        <v>10</v>
+      <c r="D41" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="E41" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="F41" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="G41" s="67" t="s">
+        <v>141</v>
+      </c>
+      <c r="H41" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="I41" s="38" t="s">
+        <v>192</v>
+      </c>
+      <c r="J41" s="38">
+        <v>1</v>
+      </c>
+      <c r="K41" s="39">
+        <f t="shared" ref="K41" si="26">J41*5</f>
+        <v>5</v>
       </c>
       <c r="L41" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M41" s="61">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="N41" s="61">
-        <f>M41*K41</f>
-        <v>0.15</v>
-      </c>
-      <c r="O41" s="36"/>
+        <v>209</v>
+      </c>
+      <c r="M41" s="62">
+        <v>0.1</v>
+      </c>
+      <c r="N41" s="62">
+        <f t="shared" ref="N41" si="27">M41*K41</f>
+        <v>0.5</v>
+      </c>
+      <c r="O41" s="38"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
@@ -3344,403 +3337,403 @@
         <v>14</v>
       </c>
       <c r="D42" s="36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E42" s="36" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F42" s="36" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G42" s="66" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="H42" s="36" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="J42" s="36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K42" s="37">
         <f>J42*5</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="L42" s="60" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="M42" s="61">
-        <v>2.5999999999999999E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="N42" s="61">
         <f>M42*K42</f>
-        <v>0.52</v>
+        <v>0.15</v>
       </c>
       <c r="O42" s="36"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
-      <c r="B43" s="56">
-        <f t="shared" si="0"/>
+      <c r="B43" s="54">
+        <f>ROW(B43) - ROW($B$9)</f>
         <v>34</v>
       </c>
-      <c r="C43" s="57" t="s">
+      <c r="C43" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D43" s="38" t="s">
-        <v>49</v>
-      </c>
-      <c r="E43" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="F43" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="G43" s="67" t="s">
-        <v>148</v>
-      </c>
-      <c r="H43" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="I43" s="38" t="s">
-        <v>200</v>
-      </c>
-      <c r="J43" s="38">
-        <v>1</v>
-      </c>
-      <c r="K43" s="39">
-        <f t="shared" ref="K43" si="28">J43*5</f>
-        <v>5</v>
+      <c r="D43" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E43" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="F43" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="G43" s="66" t="s">
+        <v>144</v>
+      </c>
+      <c r="H43" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="I43" s="36" t="s">
+        <v>195</v>
+      </c>
+      <c r="J43" s="36">
+        <v>4</v>
+      </c>
+      <c r="K43" s="37">
+        <f>J43*5</f>
+        <v>20</v>
       </c>
       <c r="L43" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M43" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N43" s="62">
-        <f t="shared" ref="N43" si="29">M43*K43</f>
-        <v>0.5</v>
-      </c>
-      <c r="O43" s="38"/>
+        <v>209</v>
+      </c>
+      <c r="M43" s="61">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="N43" s="61">
+        <f>M43*K43</f>
+        <v>0.52</v>
+      </c>
+      <c r="O43" s="36"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="54">
-        <f>ROW(B44) - ROW($B$9)</f>
+      <c r="B44" s="56">
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C44" s="55" t="s">
+      <c r="C44" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="D44" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="E44" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F44" s="36" t="s">
-        <v>113</v>
-      </c>
-      <c r="G44" s="66" t="s">
-        <v>149</v>
-      </c>
-      <c r="H44" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="I44" s="36" t="s">
-        <v>201</v>
-      </c>
-      <c r="J44" s="36">
-        <v>4</v>
-      </c>
-      <c r="K44" s="37">
-        <f>J44*5</f>
-        <v>20</v>
+      <c r="D44" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="E44" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="F44" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="G44" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="H44" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="I44" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="J44" s="38">
+        <v>1</v>
+      </c>
+      <c r="K44" s="39">
+        <f t="shared" ref="K44" si="28">J44*5</f>
+        <v>5</v>
       </c>
       <c r="L44" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M44" s="61">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="N44" s="61">
-        <f>M44*K44</f>
-        <v>0.36</v>
-      </c>
-      <c r="O44" s="36"/>
+        <v>209</v>
+      </c>
+      <c r="M44" s="62">
+        <v>0.1</v>
+      </c>
+      <c r="N44" s="62">
+        <f t="shared" ref="N44" si="29">M44*K44</f>
+        <v>0.5</v>
+      </c>
+      <c r="O44" s="38"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
-      <c r="B45" s="56">
-        <f t="shared" si="0"/>
+      <c r="B45" s="54">
+        <f>ROW(B45) - ROW($B$9)</f>
         <v>36</v>
       </c>
       <c r="C45" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D45" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="E45" s="38" t="s">
-        <v>92</v>
-      </c>
-      <c r="F45" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="G45" s="67" t="s">
-        <v>150</v>
-      </c>
-      <c r="H45" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="I45" s="38" t="s">
-        <v>202</v>
-      </c>
-      <c r="J45" s="38">
-        <v>1</v>
-      </c>
-      <c r="K45" s="39">
-        <f t="shared" ref="K45" si="30">J45*5</f>
-        <v>5</v>
+      <c r="D45" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="E45" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="F45" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="G45" s="66" t="s">
+        <v>146</v>
+      </c>
+      <c r="H45" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="I45" s="36" t="s">
+        <v>197</v>
+      </c>
+      <c r="J45" s="36">
+        <v>4</v>
+      </c>
+      <c r="K45" s="37">
+        <f>J45*5</f>
+        <v>20</v>
       </c>
       <c r="L45" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M45" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N45" s="62">
-        <f t="shared" ref="N45" si="31">M45*K45</f>
-        <v>0.5</v>
-      </c>
-      <c r="O45" s="38"/>
+        <v>209</v>
+      </c>
+      <c r="M45" s="61">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="N45" s="61">
+        <f>M45*K45</f>
+        <v>0.36</v>
+      </c>
+      <c r="O45" s="36"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="54">
-        <f>ROW(B46) - ROW($B$9)</f>
+      <c r="B46" s="56">
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C46" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D46" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="E46" s="36" t="s">
-        <v>93</v>
-      </c>
-      <c r="F46" s="36" t="s">
-        <v>113</v>
-      </c>
-      <c r="G46" s="66" t="s">
-        <v>151</v>
-      </c>
-      <c r="H46" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="I46" s="36" t="s">
-        <v>203</v>
-      </c>
-      <c r="J46" s="36">
+      <c r="D46" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="E46" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="F46" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="G46" s="67" t="s">
+        <v>147</v>
+      </c>
+      <c r="H46" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="I46" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="J46" s="38">
         <v>1</v>
       </c>
-      <c r="K46" s="37">
-        <f>J46*5</f>
+      <c r="K46" s="39">
+        <f t="shared" ref="K46" si="30">J46*5</f>
         <v>5</v>
       </c>
       <c r="L46" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M46" s="61">
+        <v>209</v>
+      </c>
+      <c r="M46" s="62">
         <v>0.1</v>
       </c>
-      <c r="N46" s="61">
-        <f>M46*K46</f>
+      <c r="N46" s="62">
+        <f t="shared" ref="N46" si="31">M46*K46</f>
         <v>0.5</v>
       </c>
-      <c r="O46" s="36"/>
+      <c r="O46" s="38"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="56">
+      <c r="B47" s="54">
+        <f>ROW(B47) - ROW($B$9)</f>
+        <v>38</v>
+      </c>
+      <c r="C47" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="E47" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="F47" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="G47" s="66" t="s">
+        <v>148</v>
+      </c>
+      <c r="H47" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="I47" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="J47" s="36">
+        <v>1</v>
+      </c>
+      <c r="K47" s="37">
+        <f>J47*5</f>
+        <v>5</v>
+      </c>
+      <c r="L47" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M47" s="61">
+        <v>0.1</v>
+      </c>
+      <c r="N47" s="61">
+        <f>M47*K47</f>
+        <v>0.5</v>
+      </c>
+      <c r="O47" s="36"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" s="1"/>
+      <c r="B48" s="56">
         <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="C47" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="D47" s="38" t="s">
+      <c r="D48" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="E47" s="38" t="s">
-        <v>223</v>
-      </c>
-      <c r="F47" s="38" t="s">
-        <v>224</v>
-      </c>
-      <c r="G47" s="38" t="s">
-        <v>225</v>
-      </c>
-      <c r="H47" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="I47" s="38" t="s">
-        <v>206</v>
-      </c>
-      <c r="J47" s="38">
+      <c r="E48" s="38" t="s">
+        <v>219</v>
+      </c>
+      <c r="F48" s="38" t="s">
+        <v>220</v>
+      </c>
+      <c r="G48" s="38" t="s">
+        <v>221</v>
+      </c>
+      <c r="H48" s="38" t="s">
+        <v>166</v>
+      </c>
+      <c r="I48" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="J48" s="38">
         <v>1</v>
       </c>
-      <c r="K47" s="39">
-        <f t="shared" ref="K47" si="32">J47*5</f>
+      <c r="K48" s="39">
+        <f t="shared" ref="K48" si="32">J48*5</f>
         <v>5</v>
       </c>
-      <c r="L47" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M47" s="62">
+      <c r="L48" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="M48" s="62">
         <v>2.97</v>
       </c>
-      <c r="N47" s="62">
-        <f t="shared" ref="N47" si="33">M47*K47</f>
+      <c r="N48" s="62">
+        <f t="shared" ref="N48" si="33">M48*K48</f>
         <v>14.850000000000001</v>
       </c>
-      <c r="O47" s="38"/>
-    </row>
-    <row r="48" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="1"/>
-      <c r="B48" s="54">
-        <f>ROW(B48) - ROW($B$9)</f>
-        <v>39</v>
-      </c>
-      <c r="C48" s="55" t="s">
-        <v>15</v>
-      </c>
-      <c r="D48" s="36" t="s">
-        <v>54</v>
-      </c>
-      <c r="E48" s="36" t="s">
-        <v>94</v>
-      </c>
-      <c r="F48" s="36" t="s">
-        <v>114</v>
-      </c>
-      <c r="G48" s="66" t="s">
-        <v>152</v>
-      </c>
-      <c r="H48" s="36" t="s">
-        <v>171</v>
-      </c>
-      <c r="I48" s="36" t="s">
-        <v>206</v>
-      </c>
-      <c r="J48" s="36">
-        <v>1</v>
-      </c>
-      <c r="K48" s="37">
-        <f>J48*5</f>
-        <v>5</v>
-      </c>
-      <c r="L48" s="60" t="s">
-        <v>218</v>
-      </c>
-      <c r="M48" s="61"/>
-      <c r="N48" s="61" t="s">
-        <v>206</v>
-      </c>
-      <c r="O48" s="36"/>
+      <c r="O48" s="38"/>
     </row>
     <row r="49" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
-      <c r="B49" s="56">
+      <c r="B49" s="54">
+        <f>ROW(B49) - ROW($B$9)</f>
+        <v>40</v>
+      </c>
+      <c r="C49" s="55" t="s">
+        <v>15</v>
+      </c>
+      <c r="D49" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="E49" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="F49" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="G49" s="66" t="s">
+        <v>149</v>
+      </c>
+      <c r="H49" s="36" t="s">
+        <v>167</v>
+      </c>
+      <c r="I49" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="J49" s="36">
+        <v>1</v>
+      </c>
+      <c r="K49" s="37">
+        <f>J49*5</f>
+        <v>5</v>
+      </c>
+      <c r="L49" s="60" t="s">
+        <v>214</v>
+      </c>
+      <c r="M49" s="61"/>
+      <c r="N49" s="61" t="s">
+        <v>202</v>
+      </c>
+      <c r="O49" s="36"/>
+    </row>
+    <row r="50" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="1"/>
+      <c r="B50" s="56">
         <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-      <c r="C49" s="57" t="s">
+        <v>41</v>
+      </c>
+      <c r="C50" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="D49" s="38" t="s">
+      <c r="D50" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="E49" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="F49" s="38" t="s">
-        <v>115</v>
-      </c>
-      <c r="G49" s="67" t="s">
-        <v>153</v>
-      </c>
-      <c r="H49" s="38" t="s">
-        <v>172</v>
-      </c>
-      <c r="I49" s="38" t="s">
-        <v>206</v>
-      </c>
-      <c r="J49" s="38">
+      <c r="E50" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="F50" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="G50" s="67" t="s">
+        <v>150</v>
+      </c>
+      <c r="H50" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="I50" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="J50" s="38">
         <v>1</v>
       </c>
-      <c r="K49" s="39">
-        <f t="shared" ref="K49" si="34">J49*5</f>
+      <c r="K50" s="39">
+        <f t="shared" ref="K50" si="34">J50*5</f>
         <v>5</v>
       </c>
-      <c r="L49" s="60" t="s">
-        <v>218</v>
-      </c>
-      <c r="M49" s="62"/>
-      <c r="N49" s="62" t="s">
-        <v>206</v>
-      </c>
-      <c r="O49" s="38"/>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50" s="1"/>
-      <c r="B50" s="54">
-        <f>ROW(B50) - ROW($B$9)</f>
-        <v>41</v>
-      </c>
-      <c r="C50" s="55" t="s">
-        <v>16</v>
-      </c>
-      <c r="D50" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="E50" s="36" t="s">
-        <v>96</v>
-      </c>
-      <c r="F50" s="36" t="s">
-        <v>116</v>
-      </c>
-      <c r="G50" s="66" t="s">
-        <v>154</v>
-      </c>
-      <c r="H50" s="36" t="s">
-        <v>173</v>
-      </c>
-      <c r="I50" s="36" t="s">
-        <v>206</v>
-      </c>
-      <c r="J50" s="36">
-        <v>1</v>
-      </c>
-      <c r="K50" s="37">
-        <f>J50*5</f>
-        <v>5</v>
-      </c>
       <c r="L50" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="M50" s="61">
-        <v>0.87</v>
-      </c>
-      <c r="N50" s="61">
-        <f>M50*K50</f>
-        <v>4.3499999999999996</v>
-      </c>
-      <c r="O50" s="36"/>
+        <v>214</v>
+      </c>
+      <c r="M50" s="62"/>
+      <c r="N50" s="62" t="s">
+        <v>202</v>
+      </c>
+      <c r="O50" s="38"/>
     </row>
     <row r="51" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
@@ -3752,22 +3745,22 @@
         <v>17</v>
       </c>
       <c r="D51" s="38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E51" s="38" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F51" s="38" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G51" s="38" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H51" s="38" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="I51" s="36" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="J51" s="38">
         <v>1</v>
@@ -3777,11 +3770,11 @@
         <v>5</v>
       </c>
       <c r="L51" s="60" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="M51" s="62"/>
       <c r="N51" s="62" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="O51" s="38"/>
     </row>
@@ -3792,27 +3785,27 @@
         <v>43</v>
       </c>
       <c r="C52" s="57" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="D52" s="38" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E52" s="38" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F52" s="38" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="G52" s="38" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="H52" s="38" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="I52" s="36" t="s">
-        <v>206</v>
-      </c>
-      <c r="J52" s="71">
+        <v>202</v>
+      </c>
+      <c r="J52" s="68">
         <v>1</v>
       </c>
       <c r="K52" s="39">
@@ -3820,15 +3813,15 @@
         <v>5</v>
       </c>
       <c r="L52" s="60" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="M52" s="62" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="N52" s="62" t="s">
-        <v>206</v>
-      </c>
-      <c r="O52" s="72"/>
+        <v>202</v>
+      </c>
+      <c r="O52" s="69"/>
     </row>
     <row r="53" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
@@ -3846,7 +3839,7 @@
       <c r="M53" s="35"/>
       <c r="N53" s="64">
         <f>SUM(N10:N51)</f>
-        <v>76.820499999999996</v>
+        <v>78.250500000000002</v>
       </c>
       <c r="O53" s="41"/>
     </row>
@@ -3866,7 +3859,7 @@
       <c r="M54" s="9"/>
       <c r="N54" s="65">
         <f>N53/5</f>
-        <v>15.364099999999999</v>
+        <v>15.6501</v>
       </c>
       <c r="O54" s="42"/>
     </row>
@@ -3884,27 +3877,27 @@
     <hyperlink ref="L16" r:id="rId6"/>
     <hyperlink ref="L18" r:id="rId7"/>
     <hyperlink ref="L19" r:id="rId8"/>
-    <hyperlink ref="L23" r:id="rId9"/>
-    <hyperlink ref="L28" r:id="rId10"/>
-    <hyperlink ref="L30" r:id="rId11"/>
-    <hyperlink ref="L31" r:id="rId12"/>
-    <hyperlink ref="L32" r:id="rId13"/>
-    <hyperlink ref="L33" r:id="rId14"/>
-    <hyperlink ref="L35" r:id="rId15"/>
-    <hyperlink ref="L36" r:id="rId16"/>
-    <hyperlink ref="L37" r:id="rId17"/>
-    <hyperlink ref="L38" r:id="rId18"/>
-    <hyperlink ref="L40" r:id="rId19"/>
-    <hyperlink ref="L41" r:id="rId20"/>
-    <hyperlink ref="L39" r:id="rId21"/>
-    <hyperlink ref="L42" r:id="rId22"/>
-    <hyperlink ref="L43" r:id="rId23"/>
-    <hyperlink ref="L44" r:id="rId24"/>
-    <hyperlink ref="L45" r:id="rId25"/>
-    <hyperlink ref="L46" r:id="rId26"/>
-    <hyperlink ref="L50" r:id="rId27"/>
-    <hyperlink ref="L25" r:id="rId28"/>
-    <hyperlink ref="L47" r:id="rId29"/>
+    <hyperlink ref="L24" r:id="rId9"/>
+    <hyperlink ref="L29" r:id="rId10"/>
+    <hyperlink ref="L31" r:id="rId11"/>
+    <hyperlink ref="L32" r:id="rId12"/>
+    <hyperlink ref="L33" r:id="rId13"/>
+    <hyperlink ref="L34" r:id="rId14"/>
+    <hyperlink ref="L36" r:id="rId15"/>
+    <hyperlink ref="L37" r:id="rId16"/>
+    <hyperlink ref="L38" r:id="rId17"/>
+    <hyperlink ref="L39" r:id="rId18"/>
+    <hyperlink ref="L41" r:id="rId19"/>
+    <hyperlink ref="L42" r:id="rId20"/>
+    <hyperlink ref="L40" r:id="rId21"/>
+    <hyperlink ref="L43" r:id="rId22"/>
+    <hyperlink ref="L44" r:id="rId23"/>
+    <hyperlink ref="L45" r:id="rId24"/>
+    <hyperlink ref="L46" r:id="rId25"/>
+    <hyperlink ref="L47" r:id="rId26"/>
+    <hyperlink ref="L26" r:id="rId27"/>
+    <hyperlink ref="L48" r:id="rId28"/>
+    <hyperlink ref="L22" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>

</xml_diff>

<commit_message>
#18 POE Injector added In Client BOM
</commit_message>
<xml_diff>
--- a/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
+++ b/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="230">
   <si>
     <t>Component list</t>
   </si>
@@ -639,18 +639,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Unit Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Total Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
     <t>Quantity (1 Board)</t>
   </si>
   <si>
@@ -663,9 +651,6 @@
     <t>EthPoE-Module-v2.0</t>
   </si>
   <si>
-    <t>Custom Supplier</t>
-  </si>
-  <si>
     <t>CONN JACK 1PORT 100 BASE-T PCB</t>
   </si>
   <si>
@@ -675,9 +660,6 @@
     <t>Abracon</t>
   </si>
   <si>
-    <t>Mouser</t>
-  </si>
-  <si>
     <t>IC POE CNTRL 1 CHANNEL 8SOIC</t>
   </si>
   <si>
@@ -721,16 +703,20 @@
   </si>
   <si>
     <t>SP0502BAHTG</t>
+  </si>
+  <si>
+    <t>POE Injector</t>
+  </si>
+  <si>
+    <t>Refrence Link</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="22" x14ac:knownFonts="1">
     <font>
@@ -913,7 +899,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1108,25 +1094,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1286,36 +1259,12 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1324,6 +1273,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1353,13 +1305,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -1667,7 +1619,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1680,13 +1632,11 @@
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="29.42578125" customWidth="1"/>
+    <col min="12" max="12" width="29.42578125" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1695,15 +1645,12 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-    </row>
-    <row r="2" spans="1:15" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+    </row>
+    <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="43"/>
@@ -1712,19 +1659,16 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="50" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="40"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L2" s="40"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="44"/>
@@ -1733,19 +1677,16 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="51" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="71"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L3" s="63"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="44"/>
@@ -1754,19 +1695,16 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="52" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="72"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L4" s="64"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="44"/>
@@ -1782,12 +1720,9 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="72"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L5" s="64"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="45"/>
@@ -1799,12 +1734,9 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="72"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L6" s="64"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="46"/>
@@ -1816,12 +1748,9 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="72"/>
-    </row>
-    <row r="8" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L7" s="64"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="47"/>
@@ -1833,12 +1762,9 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="72"/>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L8" s="64"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -1865,25 +1791,16 @@
         <v>203</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="K9" s="29" t="s">
         <v>204</v>
       </c>
       <c r="L9" s="29" t="s">
-        <v>206</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>207</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>208</v>
-      </c>
-      <c r="O9" s="29" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="54">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -1917,22 +1834,12 @@
         <f>J10*5</f>
         <v>50</v>
       </c>
-      <c r="L10" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M10" s="61">
-        <v>1.26E-2</v>
-      </c>
-      <c r="N10" s="61">
-        <f>M10*K10</f>
-        <v>0.63</v>
-      </c>
-      <c r="O10" s="36"/>
-    </row>
-    <row r="11" spans="1:15" ht="36" x14ac:dyDescent="0.25">
+      <c r="L10" s="36"/>
+    </row>
+    <row r="11" spans="1:12" ht="36" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="56">
-        <f t="shared" ref="B11:B52" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B53" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="57" t="s">
@@ -1963,18 +1870,9 @@
         <f t="shared" ref="K11" si="1">J11*5</f>
         <v>5</v>
       </c>
-      <c r="L11" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M11" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="N11" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="O11" s="38"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L11" s="38"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="54">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -1992,7 +1890,7 @@
       <c r="F12" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="G12" s="66" t="s">
+      <c r="G12" s="60" t="s">
         <v>117</v>
       </c>
       <c r="H12" s="36" t="s">
@@ -2008,19 +1906,9 @@
         <f>J12*5</f>
         <v>15</v>
       </c>
-      <c r="L12" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M12" s="61">
-        <v>7.0999999999999994E-2</v>
-      </c>
-      <c r="N12" s="61">
-        <f>M12*K12</f>
-        <v>1.0649999999999999</v>
-      </c>
-      <c r="O12" s="36"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L12" s="36"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="56">
         <f t="shared" si="0"/>
@@ -2038,7 +1926,7 @@
       <c r="F13" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="G13" s="67" t="s">
+      <c r="G13" s="61" t="s">
         <v>118</v>
       </c>
       <c r="H13" s="38" t="s">
@@ -2054,19 +1942,9 @@
         <f t="shared" ref="K13" si="2">J13*5</f>
         <v>5</v>
       </c>
-      <c r="L13" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M13" s="62">
-        <v>2.33</v>
-      </c>
-      <c r="N13" s="62">
-        <f t="shared" ref="N13" si="3">M13*K13</f>
-        <v>11.65</v>
-      </c>
-      <c r="O13" s="38"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L13" s="38"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="54">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -2084,7 +1962,7 @@
       <c r="F14" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="G14" s="66" t="s">
+      <c r="G14" s="60" t="s">
         <v>119</v>
       </c>
       <c r="H14" s="36" t="s">
@@ -2100,19 +1978,9 @@
         <f>J14*5</f>
         <v>5</v>
       </c>
-      <c r="L14" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M14" s="61">
-        <v>0.1</v>
-      </c>
-      <c r="N14" s="61">
-        <f>M14*K14</f>
-        <v>0.5</v>
-      </c>
-      <c r="O14" s="36"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L14" s="36"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="56">
         <f t="shared" si="0"/>
@@ -2130,7 +1998,7 @@
       <c r="F15" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="G15" s="66" t="s">
+      <c r="G15" s="60" t="s">
         <v>120</v>
       </c>
       <c r="H15" s="38" t="s">
@@ -2143,22 +2011,12 @@
         <v>3</v>
       </c>
       <c r="K15" s="39">
-        <f t="shared" ref="K15" si="4">J15*5</f>
+        <f t="shared" ref="K15" si="3">J15*5</f>
         <v>15</v>
       </c>
-      <c r="L15" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M15" s="62">
-        <v>5.5E-2</v>
-      </c>
-      <c r="N15" s="62">
-        <f t="shared" ref="N15" si="5">M15*K15</f>
-        <v>0.82499999999999996</v>
-      </c>
-      <c r="O15" s="38"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L15" s="38"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="54">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -2176,7 +2034,7 @@
       <c r="F16" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="G16" s="66" t="s">
+      <c r="G16" s="60" t="s">
         <v>121</v>
       </c>
       <c r="H16" s="36" t="s">
@@ -2192,19 +2050,9 @@
         <f>J16*5</f>
         <v>5</v>
       </c>
-      <c r="L16" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M16" s="61">
-        <v>0.75</v>
-      </c>
-      <c r="N16" s="61">
-        <f>M16*K16</f>
-        <v>3.75</v>
-      </c>
-      <c r="O16" s="36"/>
-    </row>
-    <row r="17" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L16" s="36"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="56">
         <f t="shared" si="0"/>
@@ -2222,7 +2070,7 @@
       <c r="F17" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="G17" s="67" t="s">
+      <c r="G17" s="61" t="s">
         <v>122</v>
       </c>
       <c r="H17" s="38" t="s">
@@ -2235,21 +2083,12 @@
         <v>2</v>
       </c>
       <c r="K17" s="39">
-        <f t="shared" ref="K17" si="6">J17*5</f>
+        <f t="shared" ref="K17" si="4">J17*5</f>
         <v>10</v>
       </c>
-      <c r="L17" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M17" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="N17" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="O17" s="38"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L17" s="38"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="54">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -2267,7 +2106,7 @@
       <c r="F18" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="G18" s="66" t="s">
+      <c r="G18" s="60" t="s">
         <v>123</v>
       </c>
       <c r="H18" s="36" t="s">
@@ -2283,19 +2122,9 @@
         <f>J18*5</f>
         <v>10</v>
       </c>
-      <c r="L18" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M18" s="61">
-        <v>9.7000000000000003E-2</v>
-      </c>
-      <c r="N18" s="61">
-        <f>M18*K18</f>
-        <v>0.97</v>
-      </c>
-      <c r="O18" s="36"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L18" s="36"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="56">
         <f t="shared" si="0"/>
@@ -2313,7 +2142,7 @@
       <c r="F19" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="G19" s="67" t="s">
+      <c r="G19" s="61" t="s">
         <v>124</v>
       </c>
       <c r="H19" s="38" t="s">
@@ -2326,22 +2155,12 @@
         <v>1</v>
       </c>
       <c r="K19" s="39">
-        <f t="shared" ref="K19" si="7">J19*5</f>
+        <f t="shared" ref="K19" si="5">J19*5</f>
         <v>5</v>
       </c>
-      <c r="L19" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M19" s="62">
-        <v>0.32</v>
-      </c>
-      <c r="N19" s="62">
-        <f t="shared" ref="N19:N22" si="8">M19*K19</f>
-        <v>1.6</v>
-      </c>
-      <c r="O19" s="38"/>
-    </row>
-    <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L19" s="38"/>
+    </row>
+    <row r="20" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="54">
         <f>ROW(B20) - ROW($B$9)</f>
@@ -2359,7 +2178,7 @@
       <c r="F20" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="G20" s="66" t="s">
+      <c r="G20" s="60" t="s">
         <v>125</v>
       </c>
       <c r="H20" s="36" t="s">
@@ -2375,14 +2194,9 @@
         <f>J20*5</f>
         <v>5</v>
       </c>
-      <c r="L20" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M20" s="61"/>
-      <c r="N20" s="62"/>
-      <c r="O20" s="36"/>
-    </row>
-    <row r="21" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L20" s="36"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="56">
         <f t="shared" si="0"/>
@@ -2400,7 +2214,7 @@
       <c r="F21" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="G21" s="67" t="s">
+      <c r="G21" s="61" t="s">
         <v>126</v>
       </c>
       <c r="H21" s="38" t="s">
@@ -2413,17 +2227,12 @@
         <v>1</v>
       </c>
       <c r="K21" s="39">
-        <f t="shared" ref="K21:K22" si="9">J21*5</f>
+        <f t="shared" ref="K21:K22" si="6">J21*5</f>
         <v>5</v>
       </c>
-      <c r="L21" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M21" s="62"/>
-      <c r="N21" s="62"/>
-      <c r="O21" s="38"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L21" s="38"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="56">
         <f t="shared" si="0"/>
@@ -2433,16 +2242,16 @@
         <v>16</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="E22" s="36" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="F22" s="36" t="s">
         <v>107</v>
       </c>
       <c r="G22" s="36" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="H22" s="36" t="s">
         <v>169</v>
@@ -2454,22 +2263,12 @@
         <v>2</v>
       </c>
       <c r="K22" s="37">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>10</v>
       </c>
-      <c r="L22" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M22" s="61">
-        <v>0.57799999999999996</v>
-      </c>
-      <c r="N22" s="62">
-        <f t="shared" si="8"/>
-        <v>5.7799999999999994</v>
-      </c>
-      <c r="O22" s="36"/>
-    </row>
-    <row r="23" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L22" s="36"/>
+    </row>
+    <row r="23" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="54">
         <f>ROW(B23) - ROW($B$9)</f>
@@ -2482,16 +2281,16 @@
         <v>31</v>
       </c>
       <c r="E23" s="36" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="F23" s="36" t="s">
         <v>103</v>
       </c>
       <c r="G23" s="36" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="H23" s="36" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="I23" s="36" t="s">
         <v>202</v>
@@ -2503,16 +2302,9 @@
         <f>J23*5</f>
         <v>5</v>
       </c>
-      <c r="L23" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M23" s="61"/>
-      <c r="N23" s="61" t="s">
-        <v>202</v>
-      </c>
-      <c r="O23" s="36"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L23" s="36"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="56">
         <f t="shared" si="0"/>
@@ -2530,7 +2322,7 @@
       <c r="F24" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="G24" s="67" t="s">
+      <c r="G24" s="61" t="s">
         <v>127</v>
       </c>
       <c r="H24" s="38" t="s">
@@ -2543,22 +2335,12 @@
         <v>2</v>
       </c>
       <c r="K24" s="39">
-        <f t="shared" ref="K24" si="10">J24*5</f>
+        <f t="shared" ref="K24" si="7">J24*5</f>
         <v>10</v>
       </c>
-      <c r="L24" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M24" s="62">
-        <v>0.38</v>
-      </c>
-      <c r="N24" s="62">
-        <f t="shared" ref="N24" si="11">M24*K24</f>
-        <v>3.8</v>
-      </c>
-      <c r="O24" s="38"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L24" s="38"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="54">
         <f>ROW(B25) - ROW($B$9)</f>
@@ -2592,18 +2374,9 @@
         <f>J25*5</f>
         <v>5</v>
       </c>
-      <c r="L25" s="36" t="s">
-        <v>202</v>
-      </c>
-      <c r="M25" s="63" t="s">
-        <v>202</v>
-      </c>
-      <c r="N25" s="63" t="s">
-        <v>202</v>
-      </c>
-      <c r="O25" s="36"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L25" s="36"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="56">
         <f t="shared" si="0"/>
@@ -2616,16 +2389,16 @@
         <v>34</v>
       </c>
       <c r="E26" s="38" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F26" s="38" t="s">
         <v>200</v>
       </c>
       <c r="G26" s="38" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="H26" s="38" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="I26" s="38" t="s">
         <v>202</v>
@@ -2634,22 +2407,12 @@
         <v>1</v>
       </c>
       <c r="K26" s="39">
-        <f t="shared" ref="K26" si="12">J26*5</f>
+        <f t="shared" ref="K26" si="8">J26*5</f>
         <v>5</v>
       </c>
-      <c r="L26" s="60" t="s">
-        <v>218</v>
-      </c>
-      <c r="M26" s="62">
-        <v>3.47</v>
-      </c>
-      <c r="N26" s="62">
-        <f t="shared" ref="N26" si="13">M26*K26</f>
-        <v>17.350000000000001</v>
-      </c>
-      <c r="O26" s="38"/>
-    </row>
-    <row r="27" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L26" s="38"/>
+    </row>
+    <row r="27" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="54">
         <f>ROW(B27) - ROW($B$9)</f>
@@ -2667,7 +2430,7 @@
       <c r="F27" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="G27" s="66" t="s">
+      <c r="G27" s="60" t="s">
         <v>128</v>
       </c>
       <c r="H27" s="36" t="s">
@@ -2683,16 +2446,9 @@
         <f>J27*5</f>
         <v>5</v>
       </c>
-      <c r="L27" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M27" s="61"/>
-      <c r="N27" s="61" t="s">
-        <v>202</v>
-      </c>
-      <c r="O27" s="36"/>
-    </row>
-    <row r="28" spans="1:15" ht="48" x14ac:dyDescent="0.25">
+      <c r="L27" s="36"/>
+    </row>
+    <row r="28" spans="1:12" ht="48" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="56">
         <f t="shared" si="0"/>
@@ -2710,7 +2466,7 @@
       <c r="F28" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="G28" s="67" t="s">
+      <c r="G28" s="61" t="s">
         <v>129</v>
       </c>
       <c r="H28" s="38" t="s">
@@ -2723,19 +2479,12 @@
         <v>1</v>
       </c>
       <c r="K28" s="39">
-        <f t="shared" ref="K28" si="14">J28*5</f>
+        <f t="shared" ref="K28" si="9">J28*5</f>
         <v>5</v>
       </c>
-      <c r="L28" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M28" s="62"/>
-      <c r="N28" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="O28" s="38"/>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L28" s="38"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="54">
         <f>ROW(B29) - ROW($B$9)</f>
@@ -2753,7 +2502,7 @@
       <c r="F29" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="G29" s="66" t="s">
+      <c r="G29" s="60" t="s">
         <v>130</v>
       </c>
       <c r="H29" s="36" t="s">
@@ -2769,19 +2518,9 @@
         <f>J29*5</f>
         <v>5</v>
       </c>
-      <c r="L29" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M29" s="61">
-        <v>0.46</v>
-      </c>
-      <c r="N29" s="61">
-        <f>M29*K29</f>
-        <v>2.3000000000000003</v>
-      </c>
-      <c r="O29" s="36"/>
-    </row>
-    <row r="30" spans="1:15" ht="36" x14ac:dyDescent="0.25">
+      <c r="L29" s="36"/>
+    </row>
+    <row r="30" spans="1:12" ht="36" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="56">
         <f t="shared" si="0"/>
@@ -2799,7 +2538,7 @@
       <c r="F30" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="G30" s="67" t="s">
+      <c r="G30" s="61" t="s">
         <v>131</v>
       </c>
       <c r="H30" s="38" t="s">
@@ -2812,19 +2551,12 @@
         <v>1</v>
       </c>
       <c r="K30" s="39">
-        <f t="shared" ref="K30" si="15">J30*5</f>
+        <f t="shared" ref="K30" si="10">J30*5</f>
         <v>5</v>
       </c>
-      <c r="L30" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M30" s="62"/>
-      <c r="N30" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="O30" s="38"/>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L30" s="38"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="54">
         <f>ROW(B31) - ROW($B$9)</f>
@@ -2842,7 +2574,7 @@
       <c r="F31" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G31" s="66" t="s">
+      <c r="G31" s="60" t="s">
         <v>132</v>
       </c>
       <c r="H31" s="36" t="s">
@@ -2858,19 +2590,9 @@
         <f>J31*5</f>
         <v>5</v>
       </c>
-      <c r="L31" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M31" s="61">
-        <v>0.2155</v>
-      </c>
-      <c r="N31" s="61">
-        <f>M31*K31</f>
-        <v>1.0774999999999999</v>
-      </c>
-      <c r="O31" s="36"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L31" s="36"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="56">
         <f t="shared" si="0"/>
@@ -2880,7 +2602,7 @@
         <v>14</v>
       </c>
       <c r="D32" s="38" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="E32" s="38" t="s">
         <v>77</v>
@@ -2888,7 +2610,7 @@
       <c r="F32" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="G32" s="67" t="s">
+      <c r="G32" s="61" t="s">
         <v>133</v>
       </c>
       <c r="H32" s="38" t="s">
@@ -2901,22 +2623,12 @@
         <v>2</v>
       </c>
       <c r="K32" s="39">
-        <f t="shared" ref="K32" si="16">J32*5</f>
+        <f t="shared" ref="K32" si="11">J32*5</f>
         <v>10</v>
       </c>
-      <c r="L32" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M32" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N32" s="62">
-        <f t="shared" ref="N32" si="17">M32*K32</f>
-        <v>1</v>
-      </c>
-      <c r="O32" s="38"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L32" s="38"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="54">
         <f>ROW(B33) - ROW($B$9)</f>
@@ -2934,7 +2646,7 @@
       <c r="F33" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="G33" s="66" t="s">
+      <c r="G33" s="60" t="s">
         <v>134</v>
       </c>
       <c r="H33" s="36" t="s">
@@ -2950,19 +2662,9 @@
         <f>J33*5</f>
         <v>5</v>
       </c>
-      <c r="L33" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M33" s="61">
-        <v>0.9</v>
-      </c>
-      <c r="N33" s="61">
-        <f>M33*K33</f>
-        <v>4.5</v>
-      </c>
-      <c r="O33" s="36"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L33" s="36"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="56">
         <f t="shared" si="0"/>
@@ -2980,7 +2682,7 @@
       <c r="F34" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="G34" s="67" t="s">
+      <c r="G34" s="61" t="s">
         <v>135</v>
       </c>
       <c r="H34" s="38" t="s">
@@ -2993,22 +2695,12 @@
         <v>1</v>
       </c>
       <c r="K34" s="39">
-        <f t="shared" ref="K34" si="18">J34*5</f>
+        <f t="shared" ref="K34" si="12">J34*5</f>
         <v>5</v>
       </c>
-      <c r="L34" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M34" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N34" s="62">
-        <f t="shared" ref="N34" si="19">M34*K34</f>
-        <v>0.5</v>
-      </c>
-      <c r="O34" s="38"/>
-    </row>
-    <row r="35" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L34" s="38"/>
+    </row>
+    <row r="35" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="54">
         <f>ROW(B35) - ROW($B$9)</f>
@@ -3026,7 +2718,7 @@
       <c r="F35" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G35" s="66" t="s">
+      <c r="G35" s="60" t="s">
         <v>136</v>
       </c>
       <c r="H35" s="36" t="s">
@@ -3042,16 +2734,9 @@
         <f>J35*5</f>
         <v>5</v>
       </c>
-      <c r="L35" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M35" s="61"/>
-      <c r="N35" s="61" t="s">
-        <v>202</v>
-      </c>
-      <c r="O35" s="36"/>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L35" s="36"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="56">
         <f t="shared" si="0"/>
@@ -3069,7 +2754,7 @@
       <c r="F36" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="G36" s="66" t="s">
+      <c r="G36" s="60" t="s">
         <v>137</v>
       </c>
       <c r="H36" s="38" t="s">
@@ -3082,22 +2767,12 @@
         <v>1</v>
       </c>
       <c r="K36" s="39">
-        <f t="shared" ref="K36" si="20">J36*5</f>
+        <f t="shared" ref="K36" si="13">J36*5</f>
         <v>5</v>
       </c>
-      <c r="L36" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M36" s="62">
-        <v>0.15</v>
-      </c>
-      <c r="N36" s="62">
-        <f t="shared" ref="N36" si="21">M36*K36</f>
-        <v>0.75</v>
-      </c>
-      <c r="O36" s="38"/>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L36" s="38"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="54">
         <f>ROW(B37) - ROW($B$9)</f>
@@ -3115,7 +2790,7 @@
       <c r="F37" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G37" s="66" t="s">
+      <c r="G37" s="60" t="s">
         <v>138</v>
       </c>
       <c r="H37" s="36" t="s">
@@ -3131,19 +2806,9 @@
         <f>J37*5</f>
         <v>5</v>
       </c>
-      <c r="L37" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M37" s="61">
-        <v>0.1</v>
-      </c>
-      <c r="N37" s="61">
-        <f>M37*K37</f>
-        <v>0.5</v>
-      </c>
-      <c r="O37" s="36"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L37" s="36"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="56">
         <f t="shared" si="0"/>
@@ -3161,7 +2826,7 @@
       <c r="F38" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="G38" s="67" t="s">
+      <c r="G38" s="61" t="s">
         <v>139</v>
       </c>
       <c r="H38" s="38" t="s">
@@ -3174,22 +2839,12 @@
         <v>1</v>
       </c>
       <c r="K38" s="39">
-        <f t="shared" ref="K38" si="22">J38*5</f>
+        <f t="shared" ref="K38" si="14">J38*5</f>
         <v>5</v>
       </c>
-      <c r="L38" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M38" s="61">
-        <v>0.1</v>
-      </c>
-      <c r="N38" s="62">
-        <f t="shared" ref="N38" si="23">M38*K38</f>
-        <v>0.5</v>
-      </c>
-      <c r="O38" s="38"/>
-    </row>
-    <row r="39" spans="1:15" ht="24" x14ac:dyDescent="0.25">
+      <c r="L38" s="38"/>
+    </row>
+    <row r="39" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="54">
         <f>ROW(B39) - ROW($B$9)</f>
@@ -3199,7 +2854,7 @@
         <v>14</v>
       </c>
       <c r="D39" s="36" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="E39" s="36" t="s">
         <v>84</v>
@@ -3207,7 +2862,7 @@
       <c r="F39" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G39" s="66" t="s">
+      <c r="G39" s="60" t="s">
         <v>140</v>
       </c>
       <c r="H39" s="36" t="s">
@@ -3223,19 +2878,9 @@
         <f>J39*5</f>
         <v>65</v>
       </c>
-      <c r="L39" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M39" s="61">
-        <v>1.6199999999999999E-2</v>
-      </c>
-      <c r="N39" s="61">
-        <f>M39*K39</f>
-        <v>1.0529999999999999</v>
-      </c>
-      <c r="O39" s="36"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L39" s="36"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="56">
         <f>ROW(B40) - ROW($B$9)</f>
@@ -3245,7 +2890,7 @@
         <v>14</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="E40" s="38" t="s">
         <v>87</v>
@@ -3253,7 +2898,7 @@
       <c r="F40" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="G40" s="67" t="s">
+      <c r="G40" s="61" t="s">
         <v>143</v>
       </c>
       <c r="H40" s="38" t="s">
@@ -3266,22 +2911,12 @@
         <v>3</v>
       </c>
       <c r="K40" s="39">
-        <f t="shared" ref="K40" si="24">J40*5</f>
+        <f t="shared" ref="K40" si="15">J40*5</f>
         <v>15</v>
       </c>
-      <c r="L40" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M40" s="62">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="N40" s="62">
-        <f t="shared" ref="N40" si="25">M40*K40</f>
-        <v>0.26999999999999996</v>
-      </c>
-      <c r="O40" s="38"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L40" s="38"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="56">
         <f t="shared" si="0"/>
@@ -3299,7 +2934,7 @@
       <c r="F41" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="G41" s="67" t="s">
+      <c r="G41" s="61" t="s">
         <v>141</v>
       </c>
       <c r="H41" s="38" t="s">
@@ -3312,22 +2947,12 @@
         <v>1</v>
       </c>
       <c r="K41" s="39">
-        <f t="shared" ref="K41" si="26">J41*5</f>
+        <f t="shared" ref="K41" si="16">J41*5</f>
         <v>5</v>
       </c>
-      <c r="L41" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M41" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N41" s="62">
-        <f t="shared" ref="N41" si="27">M41*K41</f>
-        <v>0.5</v>
-      </c>
-      <c r="O41" s="38"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L41" s="38"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="54">
         <f>ROW(B42) - ROW($B$9)</f>
@@ -3345,7 +2970,7 @@
       <c r="F42" s="36" t="s">
         <v>111</v>
       </c>
-      <c r="G42" s="66" t="s">
+      <c r="G42" s="60" t="s">
         <v>142</v>
       </c>
       <c r="H42" s="36" t="s">
@@ -3361,19 +2986,9 @@
         <f>J42*5</f>
         <v>10</v>
       </c>
-      <c r="L42" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M42" s="61">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="N42" s="61">
-        <f>M42*K42</f>
-        <v>0.15</v>
-      </c>
-      <c r="O42" s="36"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L42" s="36"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="54">
         <f>ROW(B43) - ROW($B$9)</f>
@@ -3391,7 +3006,7 @@
       <c r="F43" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="66" t="s">
+      <c r="G43" s="60" t="s">
         <v>144</v>
       </c>
       <c r="H43" s="36" t="s">
@@ -3407,19 +3022,9 @@
         <f>J43*5</f>
         <v>20</v>
       </c>
-      <c r="L43" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M43" s="61">
-        <v>2.5999999999999999E-2</v>
-      </c>
-      <c r="N43" s="61">
-        <f>M43*K43</f>
-        <v>0.52</v>
-      </c>
-      <c r="O43" s="36"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L43" s="36"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="56">
         <f t="shared" si="0"/>
@@ -3437,7 +3042,7 @@
       <c r="F44" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="G44" s="67" t="s">
+      <c r="G44" s="61" t="s">
         <v>145</v>
       </c>
       <c r="H44" s="38" t="s">
@@ -3450,22 +3055,12 @@
         <v>1</v>
       </c>
       <c r="K44" s="39">
-        <f t="shared" ref="K44" si="28">J44*5</f>
+        <f t="shared" ref="K44" si="17">J44*5</f>
         <v>5</v>
       </c>
-      <c r="L44" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M44" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N44" s="62">
-        <f t="shared" ref="N44" si="29">M44*K44</f>
-        <v>0.5</v>
-      </c>
-      <c r="O44" s="38"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L44" s="38"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="54">
         <f>ROW(B45) - ROW($B$9)</f>
@@ -3483,7 +3078,7 @@
       <c r="F45" s="36" t="s">
         <v>111</v>
       </c>
-      <c r="G45" s="66" t="s">
+      <c r="G45" s="60" t="s">
         <v>146</v>
       </c>
       <c r="H45" s="36" t="s">
@@ -3499,19 +3094,9 @@
         <f>J45*5</f>
         <v>20</v>
       </c>
-      <c r="L45" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M45" s="61">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="N45" s="61">
-        <f>M45*K45</f>
-        <v>0.36</v>
-      </c>
-      <c r="O45" s="36"/>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L45" s="36"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="56">
         <f t="shared" si="0"/>
@@ -3529,7 +3114,7 @@
       <c r="F46" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="G46" s="67" t="s">
+      <c r="G46" s="61" t="s">
         <v>147</v>
       </c>
       <c r="H46" s="38" t="s">
@@ -3542,22 +3127,12 @@
         <v>1</v>
       </c>
       <c r="K46" s="39">
-        <f t="shared" ref="K46" si="30">J46*5</f>
+        <f t="shared" ref="K46" si="18">J46*5</f>
         <v>5</v>
       </c>
-      <c r="L46" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M46" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="N46" s="62">
-        <f t="shared" ref="N46" si="31">M46*K46</f>
-        <v>0.5</v>
-      </c>
-      <c r="O46" s="38"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L46" s="38"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="54">
         <f>ROW(B47) - ROW($B$9)</f>
@@ -3575,7 +3150,7 @@
       <c r="F47" s="36" t="s">
         <v>111</v>
       </c>
-      <c r="G47" s="66" t="s">
+      <c r="G47" s="60" t="s">
         <v>148</v>
       </c>
       <c r="H47" s="36" t="s">
@@ -3591,19 +3166,9 @@
         <f>J47*5</f>
         <v>5</v>
       </c>
-      <c r="L47" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M47" s="61">
-        <v>0.1</v>
-      </c>
-      <c r="N47" s="61">
-        <f>M47*K47</f>
-        <v>0.5</v>
-      </c>
-      <c r="O47" s="36"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L47" s="36"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="56">
         <f t="shared" si="0"/>
@@ -3616,13 +3181,13 @@
         <v>53</v>
       </c>
       <c r="E48" s="38" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="F48" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="G48" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="H48" s="38" t="s">
         <v>166</v>
@@ -3634,22 +3199,12 @@
         <v>1</v>
       </c>
       <c r="K48" s="39">
-        <f t="shared" ref="K48" si="32">J48*5</f>
+        <f t="shared" ref="K48" si="19">J48*5</f>
         <v>5</v>
       </c>
-      <c r="L48" s="60" t="s">
-        <v>209</v>
-      </c>
-      <c r="M48" s="62">
-        <v>2.97</v>
-      </c>
-      <c r="N48" s="62">
-        <f t="shared" ref="N48" si="33">M48*K48</f>
-        <v>14.850000000000001</v>
-      </c>
-      <c r="O48" s="38"/>
-    </row>
-    <row r="49" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L48" s="38"/>
+    </row>
+    <row r="49" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="54">
         <f>ROW(B49) - ROW($B$9)</f>
@@ -3667,7 +3222,7 @@
       <c r="F49" s="36" t="s">
         <v>112</v>
       </c>
-      <c r="G49" s="66" t="s">
+      <c r="G49" s="60" t="s">
         <v>149</v>
       </c>
       <c r="H49" s="36" t="s">
@@ -3683,16 +3238,9 @@
         <f>J49*5</f>
         <v>5</v>
       </c>
-      <c r="L49" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M49" s="61"/>
-      <c r="N49" s="61" t="s">
-        <v>202</v>
-      </c>
-      <c r="O49" s="36"/>
-    </row>
-    <row r="50" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L49" s="36"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="56">
         <f t="shared" si="0"/>
@@ -3710,7 +3258,7 @@
       <c r="F50" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="G50" s="67" t="s">
+      <c r="G50" s="61" t="s">
         <v>150</v>
       </c>
       <c r="H50" s="38" t="s">
@@ -3723,19 +3271,12 @@
         <v>1</v>
       </c>
       <c r="K50" s="39">
-        <f t="shared" ref="K50" si="34">J50*5</f>
+        <f t="shared" ref="K50" si="20">J50*5</f>
         <v>5</v>
       </c>
-      <c r="L50" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M50" s="62"/>
-      <c r="N50" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="O50" s="38"/>
-    </row>
-    <row r="51" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="L50" s="38"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="56">
         <f t="shared" si="0"/>
@@ -3766,26 +3307,19 @@
         <v>1</v>
       </c>
       <c r="K51" s="39">
-        <f t="shared" ref="K51:K52" si="35">J51*5</f>
+        <f t="shared" ref="K51:K52" si="21">J51*5</f>
         <v>5</v>
       </c>
-      <c r="L51" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M51" s="62"/>
-      <c r="N51" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="O51" s="38"/>
-    </row>
-    <row r="52" spans="1:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L51" s="38"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="56">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
       <c r="C52" s="57" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="D52" s="38" t="s">
         <v>202</v>
@@ -3797,110 +3331,96 @@
         <v>202</v>
       </c>
       <c r="G52" s="38" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="H52" s="38" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="I52" s="36" t="s">
         <v>202</v>
       </c>
-      <c r="J52" s="68">
+      <c r="J52" s="38">
         <v>1</v>
       </c>
       <c r="K52" s="39">
-        <f t="shared" si="35"/>
+        <f t="shared" si="21"/>
         <v>5</v>
       </c>
-      <c r="L52" s="60" t="s">
-        <v>214</v>
-      </c>
-      <c r="M52" s="62" t="s">
+      <c r="L52" s="38"/>
+    </row>
+    <row r="53" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="1"/>
+      <c r="B53" s="56">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C53" s="57" t="s">
+        <v>222</v>
+      </c>
+      <c r="D53" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="N52" s="62" t="s">
+      <c r="E53" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="O52" s="69"/>
-    </row>
-    <row r="53" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="1"/>
-      <c r="B53" s="31"/>
-      <c r="C53" s="48"/>
-      <c r="D53" s="32"/>
-      <c r="E53" s="33"/>
-      <c r="F53" s="34"/>
-      <c r="G53" s="35"/>
-      <c r="H53" s="35"/>
-      <c r="I53" s="35"/>
-      <c r="J53" s="35"/>
-      <c r="K53" s="35"/>
-      <c r="L53" s="35"/>
-      <c r="M53" s="35"/>
-      <c r="N53" s="64">
-        <f>SUM(N10:N51)</f>
-        <v>78.250500000000002</v>
-      </c>
-      <c r="O53" s="41"/>
-    </row>
-    <row r="54" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F53" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="G53" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="H53" s="38"/>
+      <c r="I53" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="J53" s="38">
+        <v>1</v>
+      </c>
+      <c r="K53" s="39">
+        <v>1</v>
+      </c>
+      <c r="L53" s="65" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
-      <c r="B54" s="24"/>
-      <c r="C54" s="49"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="9"/>
-      <c r="H54" s="9"/>
-      <c r="I54" s="9"/>
-      <c r="J54" s="9"/>
-      <c r="K54" s="9"/>
-      <c r="L54" s="9"/>
-      <c r="M54" s="9"/>
-      <c r="N54" s="65">
-        <f>N53/5</f>
-        <v>15.6501</v>
-      </c>
-      <c r="O54" s="42"/>
+      <c r="B54" s="31"/>
+      <c r="C54" s="48"/>
+      <c r="D54" s="32"/>
+      <c r="E54" s="33"/>
+      <c r="F54" s="34"/>
+      <c r="G54" s="35"/>
+      <c r="H54" s="35"/>
+      <c r="I54" s="35"/>
+      <c r="J54" s="35"/>
+      <c r="K54" s="35"/>
+      <c r="L54" s="41"/>
+    </row>
+    <row r="55" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="1"/>
+      <c r="B55" s="24"/>
+      <c r="C55" s="49"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
+      <c r="I55" s="9"/>
+      <c r="J55" s="9"/>
+      <c r="K55" s="9"/>
+      <c r="L55" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="O3:O8"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="L3:L8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="L10" r:id="rId1"/>
-    <hyperlink ref="L12" r:id="rId2"/>
-    <hyperlink ref="L13" r:id="rId3"/>
-    <hyperlink ref="L14" r:id="rId4"/>
-    <hyperlink ref="L15" r:id="rId5"/>
-    <hyperlink ref="L16" r:id="rId6"/>
-    <hyperlink ref="L18" r:id="rId7"/>
-    <hyperlink ref="L19" r:id="rId8"/>
-    <hyperlink ref="L24" r:id="rId9"/>
-    <hyperlink ref="L29" r:id="rId10"/>
-    <hyperlink ref="L31" r:id="rId11"/>
-    <hyperlink ref="L32" r:id="rId12"/>
-    <hyperlink ref="L33" r:id="rId13"/>
-    <hyperlink ref="L34" r:id="rId14"/>
-    <hyperlink ref="L36" r:id="rId15"/>
-    <hyperlink ref="L37" r:id="rId16"/>
-    <hyperlink ref="L38" r:id="rId17"/>
-    <hyperlink ref="L39" r:id="rId18"/>
-    <hyperlink ref="L41" r:id="rId19"/>
-    <hyperlink ref="L42" r:id="rId20"/>
-    <hyperlink ref="L40" r:id="rId21"/>
-    <hyperlink ref="L43" r:id="rId22"/>
-    <hyperlink ref="L44" r:id="rId23"/>
-    <hyperlink ref="L45" r:id="rId24"/>
-    <hyperlink ref="L46" r:id="rId25"/>
-    <hyperlink ref="L47" r:id="rId26"/>
-    <hyperlink ref="L26" r:id="rId27"/>
-    <hyperlink ref="L48" r:id="rId28"/>
-    <hyperlink ref="L22" r:id="rId29"/>
+    <hyperlink ref="L53" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
-  <drawing r:id="rId31"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#18 eSpark BOM periperal added
</commit_message>
<xml_diff>
--- a/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
+++ b/Design Files/EthPoE-Module-v2.0/BOM/Client_BOM_EthPoE-Module-v2.0.xlsx
@@ -1265,6 +1265,9 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1273,9 +1276,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1645,10 +1645,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1684,7 +1684,7 @@
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="63"/>
+      <c r="L3" s="64"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1702,7 +1702,7 @@
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="64"/>
+      <c r="L4" s="65"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1720,7 +1720,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="64"/>
+      <c r="L5" s="65"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1734,7 +1734,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="64"/>
+      <c r="L6" s="65"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1748,7 +1748,7 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="64"/>
+      <c r="L7" s="65"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1762,7 +1762,7 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="64"/>
+      <c r="L8" s="65"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3379,7 +3379,7 @@
       <c r="K53" s="39">
         <v>1</v>
       </c>
-      <c r="L53" s="65" t="s">
+      <c r="L53" s="62" t="s">
         <v>229</v>
       </c>
     </row>

</xml_diff>